<commit_message>
docs: CIOC v3.0 permanently frozen — nomenclature, claim scope, H-new2 role, discordance flags in evidence matrix (membership unchanged)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/core_oncofetal/results/Core_oncofetal_gate_statistics_public.xlsx
+++ b/core_oncofetal/results/Core_oncofetal_gate_statistics_public.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,8 +46,14 @@
       <name val="Arial"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +83,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF7C80"/>
       </patternFill>
     </fill>
     <fill>
@@ -116,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -139,10 +150,13 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -510,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R32"/>
+  <dimension ref="A1:T32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -531,6 +545,8 @@
     <col width="20" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="60" customHeight="1">
@@ -621,6 +637,16 @@
       </c>
       <c r="R1" s="2" t="inlineStr">
         <is>
+          <t>H statistical support from</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>DISCORDANCE flags (reported, not selecting)</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
           <t>Developmental intersection (HGCA &amp; GSE230581)</t>
         </is>
       </c>
@@ -707,6 +733,16 @@
       </c>
       <c r="R2" s="4" t="inlineStr">
         <is>
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="S2" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="T2" s="4" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
@@ -791,7 +827,17 @@
           <t>-0.00 (FDR 0.99)</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="S3" s="8" t="inlineStr">
+        <is>
+          <t>Gao opposite (-0.16)</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -842,7 +888,7 @@
           <t>-0.10 (FDR 0.86)</t>
         </is>
       </c>
-      <c r="K4" s="8" t="inlineStr">
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -878,6 +924,16 @@
         </is>
       </c>
       <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-2.38); H-new2 opposite (-0.93); Gao opposite (-0.10)</t>
+        </is>
+      </c>
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -963,7 +1019,17 @@
           <t>-2.31 (FDR 1e-36)*</t>
         </is>
       </c>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>TCGA bulk significantly tumour-low (-2.31)</t>
+        </is>
+      </c>
+      <c r="T5" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -1024,7 +1090,7 @@
           <t>-1.22 (FDR 0.014)*</t>
         </is>
       </c>
-      <c r="M6" s="8" t="inlineStr">
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1050,6 +1116,16 @@
         </is>
       </c>
       <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="S6" s="8" t="inlineStr">
+        <is>
+          <t>GSE44433 significantly adult-high (-2.63)</t>
+        </is>
+      </c>
+      <c r="T6" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1135,7 +1211,17 @@
           <t>-0.33 (FDR 0.0056)*</t>
         </is>
       </c>
-      <c r="R7" s="5" t="inlineStr">
+      <c r="R7" s="4" t="inlineStr">
+        <is>
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="S7" s="8" t="inlineStr">
+        <is>
+          <t>TCGA bulk significantly tumour-low (-0.33)</t>
+        </is>
+      </c>
+      <c r="T7" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -1186,7 +1272,7 @@
           <t>NA (no one2one orthologue)</t>
         </is>
       </c>
-      <c r="K8" s="9" t="inlineStr">
+      <c r="K8" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -1196,7 +1282,7 @@
           <t>NA (not measured)</t>
         </is>
       </c>
-      <c r="M8" s="9" t="inlineStr">
+      <c r="M8" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -1222,6 +1308,16 @@
         </is>
       </c>
       <c r="R8" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S8" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="T8" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1272,7 +1368,7 @@
           <t>-0.01 (FDR 0.83)</t>
         </is>
       </c>
-      <c r="K9" s="8" t="inlineStr">
+      <c r="K9" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1307,7 +1403,17 @@
           <t>+3.88 (FDR 6.3e-18)**</t>
         </is>
       </c>
-      <c r="R9" s="5" t="inlineStr">
+      <c r="R9" s="4" t="inlineStr">
+        <is>
+          <t>HGCA</t>
+        </is>
+      </c>
+      <c r="S9" s="8" t="inlineStr">
+        <is>
+          <t>Gao opposite (-0.01)</t>
+        </is>
+      </c>
+      <c r="T9" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -1334,7 +1440,7 @@
       <c r="F10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1354,7 +1460,7 @@
           <t>-0.01 (FDR 0.77)</t>
         </is>
       </c>
-      <c r="K10" s="9" t="inlineStr">
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -1364,7 +1470,7 @@
           <t>NA (no one2one orthologue)</t>
         </is>
       </c>
-      <c r="M10" s="9" t="inlineStr">
+      <c r="M10" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -1390,6 +1496,16 @@
         </is>
       </c>
       <c r="R10" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S10" s="8" t="inlineStr">
+        <is>
+          <t>Gao opposite (-0.01)</t>
+        </is>
+      </c>
+      <c r="T10" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1440,7 +1556,7 @@
           <t>-0.58 (FDR 0.93)</t>
         </is>
       </c>
-      <c r="K11" s="8" t="inlineStr">
+      <c r="K11" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1450,7 +1566,7 @@
           <t>-0.94 (FDR 0.06)</t>
         </is>
       </c>
-      <c r="M11" s="8" t="inlineStr">
+      <c r="M11" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1476,6 +1592,16 @@
         </is>
       </c>
       <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S11" s="8" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-2.49); Gao opposite (-0.58)</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1506,7 +1632,7 @@
       <c r="F12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1526,7 +1652,7 @@
           <t>NA (not measured)</t>
         </is>
       </c>
-      <c r="K12" s="8" t="inlineStr">
+      <c r="K12" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1562,6 +1688,16 @@
         </is>
       </c>
       <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S12" s="8" t="inlineStr">
+        <is>
+          <t>H-new2 opposite (-1.08)</t>
+        </is>
+      </c>
+      <c r="T12" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1649,6 +1785,16 @@
       </c>
       <c r="R13" s="4" t="inlineStr">
         <is>
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
@@ -1735,6 +1881,16 @@
       </c>
       <c r="R14" s="4" t="inlineStr">
         <is>
+          <t>H-new2, Gao</t>
+        </is>
+      </c>
+      <c r="S14" s="8" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-0.36)</t>
+        </is>
+      </c>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
@@ -1784,7 +1940,7 @@
           <t>-1.08 (FDR 0.3)</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -1794,7 +1950,7 @@
           <t>NA (not measured)</t>
         </is>
       </c>
-      <c r="M15" s="9" t="inlineStr">
+      <c r="M15" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -1820,6 +1976,16 @@
         </is>
       </c>
       <c r="R15" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S15" s="8" t="inlineStr">
+        <is>
+          <t>Gao opposite (-1.08)</t>
+        </is>
+      </c>
+      <c r="T15" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1870,7 +2036,7 @@
           <t>-0.01 (FDR 0.98)</t>
         </is>
       </c>
-      <c r="K16" s="8" t="inlineStr">
+      <c r="K16" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1880,7 +2046,7 @@
           <t>+0.46 (FDR 0.094)</t>
         </is>
       </c>
-      <c r="M16" s="8" t="inlineStr">
+      <c r="M16" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1906,6 +2072,16 @@
         </is>
       </c>
       <c r="R16" s="4" t="inlineStr">
+        <is>
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="S16" s="8" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-0.01); Gao opposite (-0.01)</t>
+        </is>
+      </c>
+      <c r="T16" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -1956,7 +2132,7 @@
           <t>-0.41 (FDR 0.97)</t>
         </is>
       </c>
-      <c r="K17" s="9" t="inlineStr">
+      <c r="K17" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -1966,7 +2142,7 @@
           <t>NA (not measured)</t>
         </is>
       </c>
-      <c r="M17" s="9" t="inlineStr">
+      <c r="M17" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -1992,6 +2168,16 @@
         </is>
       </c>
       <c r="R17" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S17" s="8" t="inlineStr">
+        <is>
+          <t>Gao opposite (-0.41); TCGA bulk significantly tumour-low (-1.03)</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2018,7 +2204,7 @@
       <c r="F18" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="8" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2073,7 +2259,17 @@
           <t>+1.57 (FDR 7e-07)**</t>
         </is>
       </c>
-      <c r="R18" s="5" t="inlineStr">
+      <c r="R18" s="4" t="inlineStr">
+        <is>
+          <t>HGCA, Gao</t>
+        </is>
+      </c>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -2124,7 +2320,7 @@
           <t>-2.99 (FDR 0.0093)*</t>
         </is>
       </c>
-      <c r="K19" s="8" t="inlineStr">
+      <c r="K19" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2160,6 +2356,16 @@
         </is>
       </c>
       <c r="R19" s="4" t="inlineStr">
+        <is>
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="S19" s="8" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-3.60); Gao opposite (-2.99); GSE44433 significantly adult-high (-4.17)</t>
+        </is>
+      </c>
+      <c r="T19" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2247,6 +2453,16 @@
       </c>
       <c r="R20" s="4" t="inlineStr">
         <is>
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="S20" s="8" t="inlineStr">
+        <is>
+          <t>Gao opposite (-1.04); GSE44433 significantly adult-high (-3.02)</t>
+        </is>
+      </c>
+      <c r="T20" s="4" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
@@ -2276,7 +2492,7 @@
       <c r="F21" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="8" t="inlineStr">
+      <c r="G21" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2296,7 +2512,7 @@
           <t>-0.84 (FDR 0.61)</t>
         </is>
       </c>
-      <c r="K21" s="8" t="inlineStr">
+      <c r="K21" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2306,7 +2522,7 @@
           <t>-3.26 (FDR 2.6e-09)*</t>
         </is>
       </c>
-      <c r="M21" s="8" t="inlineStr">
+      <c r="M21" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2332,6 +2548,16 @@
         </is>
       </c>
       <c r="R21" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S21" s="8" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-3.87); H-new2 opposite (-3.92); Gao opposite (-0.84); GSE44433 significantly adult-high (-0.63)</t>
+        </is>
+      </c>
+      <c r="T21" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2362,7 +2588,7 @@
       <c r="F22" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="8" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2382,7 +2608,7 @@
           <t>+0.91 (FDR 0.54)</t>
         </is>
       </c>
-      <c r="K22" s="8" t="inlineStr">
+      <c r="K22" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2418,6 +2644,16 @@
         </is>
       </c>
       <c r="R22" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S22" s="8" t="inlineStr">
+        <is>
+          <t>H-new2 opposite (-0.24)</t>
+        </is>
+      </c>
+      <c r="T22" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2448,7 +2684,7 @@
       <c r="F23" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="8" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2504,6 +2740,16 @@
         </is>
       </c>
       <c r="R23" s="4" t="inlineStr">
+        <is>
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="S23" s="8" t="inlineStr">
+        <is>
+          <t>TCGA bulk significantly tumour-low (-0.46)</t>
+        </is>
+      </c>
+      <c r="T23" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2564,7 +2810,7 @@
           <t>+0.01 (FDR 0.98)</t>
         </is>
       </c>
-      <c r="M24" s="8" t="inlineStr">
+      <c r="M24" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2590,6 +2836,16 @@
         </is>
       </c>
       <c r="R24" s="4" t="inlineStr">
+        <is>
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="S24" s="8" t="inlineStr">
+        <is>
+          <t>Gao opposite (-1.54)</t>
+        </is>
+      </c>
+      <c r="T24" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2640,7 +2896,7 @@
           <t>-0.80 (FDR 0.87)</t>
         </is>
       </c>
-      <c r="K25" s="8" t="inlineStr">
+      <c r="K25" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2650,7 +2906,7 @@
           <t>NA (not measured)</t>
         </is>
       </c>
-      <c r="M25" s="9" t="inlineStr">
+      <c r="M25" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -2676,6 +2932,16 @@
         </is>
       </c>
       <c r="R25" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S25" s="8" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-5.82); H-new2 opposite (-4.26); Gao opposite (-0.80)</t>
+        </is>
+      </c>
+      <c r="T25" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2736,7 +3002,7 @@
           <t>NA (not measured)</t>
         </is>
       </c>
-      <c r="M26" s="9" t="inlineStr">
+      <c r="M26" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -2762,6 +3028,16 @@
         </is>
       </c>
       <c r="R26" s="4" t="inlineStr">
+        <is>
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="S26" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="T26" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2792,7 +3068,7 @@
       <c r="F27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="8" t="inlineStr">
+      <c r="G27" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2812,7 +3088,7 @@
           <t>NA (no one2one orthologue)</t>
         </is>
       </c>
-      <c r="K27" s="9" t="inlineStr">
+      <c r="K27" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -2822,7 +3098,7 @@
           <t>-6.51 (FDR 5.6e-06)*</t>
         </is>
       </c>
-      <c r="M27" s="8" t="inlineStr">
+      <c r="M27" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2848,6 +3124,16 @@
         </is>
       </c>
       <c r="R27" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S27" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="T27" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2878,7 +3164,7 @@
       <c r="F28" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G28" s="8" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2898,7 +3184,7 @@
           <t>+0.13 (FDR 0.77)</t>
         </is>
       </c>
-      <c r="K28" s="8" t="inlineStr">
+      <c r="K28" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2934,6 +3220,16 @@
         </is>
       </c>
       <c r="R28" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S28" s="8" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-5.05); GSE44433 significantly adult-high (-2.37); TCGA bulk significantly tumour-low (-1.75)</t>
+        </is>
+      </c>
+      <c r="T28" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2964,7 +3260,7 @@
       <c r="F29" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G29" s="8" t="inlineStr">
+      <c r="G29" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2994,7 +3290,7 @@
           <t>-0.07 (FDR 0.63)</t>
         </is>
       </c>
-      <c r="M29" s="8" t="inlineStr">
+      <c r="M29" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3020,6 +3316,16 @@
         </is>
       </c>
       <c r="R29" s="4" t="inlineStr">
+        <is>
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="S29" s="8" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-1.07)</t>
+        </is>
+      </c>
+      <c r="T29" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -3050,7 +3356,7 @@
       <c r="F30" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G30" s="8" t="inlineStr">
+      <c r="G30" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3070,7 +3376,7 @@
           <t>+0.12 (FDR 0.97)</t>
         </is>
       </c>
-      <c r="K30" s="9" t="inlineStr">
+      <c r="K30" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
@@ -3080,7 +3386,7 @@
           <t>-2.83 (FDR 1.6e-05)*</t>
         </is>
       </c>
-      <c r="M30" s="8" t="inlineStr">
+      <c r="M30" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3106,6 +3412,16 @@
         </is>
       </c>
       <c r="R30" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S30" s="8" t="inlineStr">
+        <is>
+          <t>GSE44433 significantly adult-high (-1.09)</t>
+        </is>
+      </c>
+      <c r="T30" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -3136,7 +3452,7 @@
       <c r="F31" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G31" s="8" t="inlineStr">
+      <c r="G31" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3166,7 +3482,7 @@
           <t>-4.97 (FDR 8.1e-10)*</t>
         </is>
       </c>
-      <c r="M31" s="8" t="inlineStr">
+      <c r="M31" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3192,6 +3508,16 @@
         </is>
       </c>
       <c r="R31" s="4" t="inlineStr">
+        <is>
+          <t>HGCA</t>
+        </is>
+      </c>
+      <c r="S31" s="8" t="inlineStr">
+        <is>
+          <t>GSE44433 significantly adult-high (-3.76); TCGA bulk significantly tumour-low (-1.27)</t>
+        </is>
+      </c>
+      <c r="T31" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -3218,7 +3544,7 @@
       <c r="F32" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G32" s="8" t="inlineStr">
+      <c r="G32" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3238,7 +3564,7 @@
           <t>-1.75 (FDR 0.26)</t>
         </is>
       </c>
-      <c r="K32" s="8" t="inlineStr">
+      <c r="K32" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3248,7 +3574,7 @@
           <t>+0.05 (FDR 0.89)</t>
         </is>
       </c>
-      <c r="M32" s="8" t="inlineStr">
+      <c r="M32" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3274,6 +3600,16 @@
         </is>
       </c>
       <c r="R32" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="S32" s="8" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-2.68); H-new2 opposite (-0.30); Gao opposite (-1.75)</t>
+        </is>
+      </c>
+      <c r="T32" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -4497,7 +4833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4518,6 +4854,8 @@
     <col width="20" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="60" customHeight="1">
@@ -4608,6 +4946,16 @@
       </c>
       <c r="R1" s="2" t="inlineStr">
         <is>
+          <t>H statistical support from</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>DISCORDANCE flags (reported, not selecting)</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
           <t>Developmental intersection (HGCA &amp; GSE230581)</t>
         </is>
       </c>
@@ -4692,7 +5040,17 @@
           <t>-0.00 (FDR 0.99)</t>
         </is>
       </c>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="S2" s="8" t="inlineStr">
+        <is>
+          <t>Gao opposite (-0.16)</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -4778,7 +5136,17 @@
           <t>-2.31 (FDR 1e-36)*</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="S3" s="8" t="inlineStr">
+        <is>
+          <t>TCGA bulk significantly tumour-low (-2.31)</t>
+        </is>
+      </c>
+      <c r="T3" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -4864,7 +5232,17 @@
           <t>-0.33 (FDR 0.0056)*</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
+        <is>
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="S4" s="8" t="inlineStr">
+        <is>
+          <t>TCGA bulk significantly tumour-low (-0.33)</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -4915,7 +5293,7 @@
           <t>-0.01 (FDR 0.83)</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="K5" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -4950,7 +5328,17 @@
           <t>+3.88 (FDR 6.3e-18)**</t>
         </is>
       </c>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>HGCA</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>Gao opposite (-0.01)</t>
+        </is>
+      </c>
+      <c r="T5" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -4977,7 +5365,7 @@
       <c r="F6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -5032,7 +5420,17 @@
           <t>+1.57 (FDR 7e-07)**</t>
         </is>
       </c>
-      <c r="R6" s="5" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>HGCA, Gao</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -5729,7 +6127,7 @@
       <c r="N10" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O10" s="8" t="inlineStr">
+      <c r="O10" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -5849,7 +6247,7 @@
       <c r="N12" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O12" s="8" t="inlineStr">
+      <c r="O12" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -6225,7 +6623,7 @@
       <c r="N18" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O18" s="8" t="inlineStr">
+      <c r="O18" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -6405,7 +6803,7 @@
       <c r="N21" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O21" s="8" t="inlineStr">
+      <c r="O21" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -6465,7 +6863,7 @@
       <c r="N22" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O22" s="8" t="inlineStr">
+      <c r="O22" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -6529,7 +6927,7 @@
       <c r="N23" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O23" s="8" t="inlineStr">
+      <c r="O23" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -6773,7 +7171,7 @@
       <c r="N27" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O27" s="8" t="inlineStr">
+      <c r="O27" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -6833,7 +7231,7 @@
       <c r="N28" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O28" s="8" t="inlineStr">
+      <c r="O28" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -6893,7 +7291,7 @@
       <c r="N29" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O29" s="8" t="inlineStr">
+      <c r="O29" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -6957,7 +7355,7 @@
       <c r="N30" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O30" s="8" t="inlineStr">
+      <c r="O30" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -7021,7 +7419,7 @@
       <c r="N31" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O31" s="8" t="inlineStr">
+      <c r="O31" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -7077,7 +7475,7 @@
       <c r="N32" s="4" t="b">
         <v>0</v>
       </c>
-      <c r="O32" s="8" t="inlineStr">
+      <c r="O32" s="9" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -22401,7 +22799,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22497,58 +22895,88 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Core (v3.0)</t>
+          <t>Conserved Intestinal Oncofetal Core (CIOC), v3.0, permanently frozen</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr"/>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>L &amp; H &amp; M &amp; C all pass</t>
+          <t>L &amp; H &amp; M &amp; C all pass. Operational definition: literature-anchored genes with replicated developmental evidence and malignant epithelial reactivation; not a fetal-specific marker set</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Stringent intersection set (v1.0)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>sensitivity</t>
-        </is>
-      </c>
+          <t>H wording</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr"/>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>HGCA &gt;=9 PCW &amp; GSE230581 &amp; Joanito &amp; Pelka each log2FC &gt;= 0.5 &amp; FDR &lt; 0.05 (not measured = NE)</t>
+          <t>concordant fetal enrichment across &gt;= 2 independent comparisons, statistical support in &gt;= 1; H-new2 (cross-study) serves as a statistical-support dataset, direction is evaluated with HGCA and Gao; all three log2FC shown</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Cell notation</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr"/>
+          <t>Discordance flags</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>reported, never selecting</t>
+        </is>
+      </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>log2FC (FDR); ** log2FC &gt;= 0.5 &amp; FDR &lt; 0.05; * FDR &lt; 0.05 below effect threshold; NA = not measured / no orthologue</t>
+          <t>human contrast in opposite direction; GSE44433 significantly adult-high; TCGA bulk significantly tumour-low</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>Sensitivity analysis using single-dataset hard intersections (former v1.0)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>sensitivity only; not an alternative Core</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>HGCA &gt;=9 PCW &amp; GSE230581 &amp; Joanito &amp; Pelka each log2FC &gt;= 0.5 &amp; FDR &lt; 0.05 (not measured = NE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Cell notation</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>log2FC (FDR); ** log2FC &gt;= 0.5 &amp; FDR &lt; 0.05; * FDR &lt; 0.05 below effect threshold; NA = not measured / no orthologue</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
           <t>Supportive evidence</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>never selecting</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>GSE44433, TCGA, Pikkupeura cultures, HGCA all fetal, Joanito sensitivity, Pelka P</t>
         </is>

</xml_diff>

<commit_message>
fix: evaluate 31 panel genes without genome-wide expression filter; explicit NA provenance; rebuilt CIOC evidence matrix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/core_oncofetal/results/Core_oncofetal_gate_statistics_public.xlsx
+++ b/core_oncofetal/results/Core_oncofetal_gate_statistics_public.xlsx
@@ -82,17 +82,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDEDED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FF7C80"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
       </patternFill>
     </fill>
     <fill>
@@ -147,10 +147,10 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -714,7 +714,7 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>+7.78 (FDR 0.0017)**</t>
+          <t>+7.78 (FDR 0.0016)**</t>
         </is>
       </c>
       <c r="N2" s="6" t="inlineStr">
@@ -833,9 +833,9 @@
           <t>concordant</t>
         </is>
       </c>
-      <c r="Q3" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>+3.89 (FDR 9.3e-06)** [low count]</t>
         </is>
       </c>
       <c r="R3" s="4" t="inlineStr">
@@ -848,7 +848,7 @@
           <t>HGCA, H-new2</t>
         </is>
       </c>
-      <c r="T3" s="8" t="inlineStr">
+      <c r="T3" s="7" t="inlineStr">
         <is>
           <t>Gao opposite (-0.16)</t>
         </is>
@@ -909,7 +909,7 @@
           <t>-0.10 (FDR 0.86)</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="L4" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -949,7 +949,7 @@
           <t>none</t>
         </is>
       </c>
-      <c r="T4" s="8" t="inlineStr">
+      <c r="T4" s="7" t="inlineStr">
         <is>
           <t>HGCA opposite (-2.38); H-new2 opposite (-0.93); Gao opposite (-0.10)</t>
         </is>
@@ -1050,7 +1050,7 @@
           <t>HGCA, H-new2</t>
         </is>
       </c>
-      <c r="T5" s="8" t="inlineStr">
+      <c r="T5" s="7" t="inlineStr">
         <is>
           <t>TCGA bulk significantly tumour-low (-2.31)</t>
         </is>
@@ -1121,7 +1121,7 @@
           <t>-1.22 (FDR 0.014)*</t>
         </is>
       </c>
-      <c r="N6" s="9" t="inlineStr">
+      <c r="N6" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1151,7 +1151,7 @@
           <t>HGCA, H-new2</t>
         </is>
       </c>
-      <c r="T6" s="8" t="inlineStr">
+      <c r="T6" s="7" t="inlineStr">
         <is>
           <t>GSE44433 significantly adult-high (-2.63)</t>
         </is>
@@ -1252,7 +1252,7 @@
           <t>HGCA, H-new2</t>
         </is>
       </c>
-      <c r="T7" s="8" t="inlineStr">
+      <c r="T7" s="7" t="inlineStr">
         <is>
           <t>TCGA bulk significantly tumour-low (-0.33)</t>
         </is>
@@ -1298,19 +1298,19 @@
           <t>Mustata et al., Cell Reports, 2013; Nusse et al., Nature, 2018; Yui et al., Cell Stem Cell, 2018 | Chen et al., Cell Stem Cell, 2023; Cheung et al., Cell Stem Cell, 2020; Karo-Atar et al., Journal of Experimental Medicine, 2022; Nusse et al., Nature, 2018; Yui et al., Cell Stem Cell, 2018</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="J8" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="K8" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
         </is>
       </c>
       <c r="L8" s="10" t="inlineStr">
@@ -1318,34 +1318,34 @@
           <t>NE</t>
         </is>
       </c>
-      <c r="M8" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="N8" s="10" t="inlineStr">
-        <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="O8" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="P8" s="7" t="inlineStr">
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>-2.26 (FDR 0.011)*</t>
+        </is>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="O8" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="P8" s="9" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="Q8" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="R8" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="R8" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
         </is>
       </c>
       <c r="S8" s="4" t="inlineStr">
@@ -1404,9 +1404,9 @@
           <t>+2.52 (FDR 0.029)**</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>+7.30 (FDR 0.0021)**</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1414,9 +1414,9 @@
           <t>-0.01 (FDR 0.83)</t>
         </is>
       </c>
-      <c r="L9" s="9" t="inlineStr">
-        <is>
-          <t>fail</t>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>pass</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
@@ -1451,10 +1451,10 @@
       </c>
       <c r="S9" s="4" t="inlineStr">
         <is>
-          <t>HGCA</t>
-        </is>
-      </c>
-      <c r="T9" s="8" t="inlineStr">
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="T9" s="7" t="inlineStr">
         <is>
           <t>Gao opposite (-0.01)</t>
         </is>
@@ -1500,14 +1500,14 @@
           <t>none identified</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>-1.43 (FDR 0.38) [low count]</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>NA (zero_expression)</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -1515,34 +1515,34 @@
           <t>-0.01 (FDR 0.77)</t>
         </is>
       </c>
-      <c r="L10" s="10" t="inlineStr">
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="M10" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="N10" s="10" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="M10" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="N10" s="10" t="inlineStr">
-        <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="O10" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="P10" s="7" t="inlineStr">
+      <c r="O10" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="P10" s="9" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="Q10" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="Q10" s="4" t="inlineStr">
+        <is>
+          <t>+5.08 (FDR 0.0044)** [low count]</t>
         </is>
       </c>
       <c r="R10" s="5" t="inlineStr">
@@ -1555,9 +1555,9 @@
           <t>none</t>
         </is>
       </c>
-      <c r="T10" s="8" t="inlineStr">
-        <is>
-          <t>Gao opposite (-0.01)</t>
+      <c r="T10" s="7" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-1.43); Gao opposite (-0.01)</t>
         </is>
       </c>
       <c r="U10" s="4" t="inlineStr">
@@ -1606,9 +1606,9 @@
           <t>-2.49 (FDR 0.0038)*</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>+1.22 (FDR 0.049)** [low count]</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
@@ -1616,7 +1616,7 @@
           <t>-0.58 (FDR 0.93)</t>
         </is>
       </c>
-      <c r="L11" s="9" t="inlineStr">
+      <c r="L11" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1626,7 +1626,7 @@
           <t>-0.94 (FDR 0.06)</t>
         </is>
       </c>
-      <c r="N11" s="9" t="inlineStr">
+      <c r="N11" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -1653,10 +1653,10 @@
       </c>
       <c r="S11" s="4" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="T11" s="8" t="inlineStr">
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
         <is>
           <t>HGCA opposite (-2.49); Gao opposite (-0.58)</t>
         </is>
@@ -1712,19 +1712,19 @@
           <t>-1.08 (FDR 0.017)*</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="L12" s="9" t="inlineStr">
+      <c r="K12" s="9" t="inlineStr">
+        <is>
+          <t>NA (not_available_in_source)</t>
+        </is>
+      </c>
+      <c r="L12" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>+1.03 (FDR 0.00068)**</t>
+          <t>+1.03 (FDR 0.00067)**</t>
         </is>
       </c>
       <c r="N12" s="6" t="inlineStr">
@@ -1732,12 +1732,12 @@
           <t>pass</t>
         </is>
       </c>
-      <c r="O12" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="P12" s="7" t="inlineStr">
+      <c r="O12" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="P12" s="9" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1757,7 +1757,7 @@
           <t>none</t>
         </is>
       </c>
-      <c r="T12" s="8" t="inlineStr">
+      <c r="T12" s="7" t="inlineStr">
         <is>
           <t>H-new2 opposite (-1.08)</t>
         </is>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>+6.37 (FDR 5.6e-06)**</t>
+          <t>+6.37 (FDR 5.7e-06)**</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -1934,12 +1934,12 @@
           <t>pass</t>
         </is>
       </c>
-      <c r="O14" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="P14" s="7" t="inlineStr">
+      <c r="O14" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="P14" s="9" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -1959,7 +1959,7 @@
           <t>H-new2, Gao</t>
         </is>
       </c>
-      <c r="T14" s="8" t="inlineStr">
+      <c r="T14" s="7" t="inlineStr">
         <is>
           <t>HGCA opposite (-0.36)</t>
         </is>
@@ -2005,14 +2005,14 @@
           <t>Pikkupeura et al., Science Advances, 2023 | Hartl et al., Sci Adv, 2024; Yui et al., Cell Stem Cell, 2018</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="J15" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>+5.63 (FDR 0.003)** [low count]</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>+4.46 (FDR 0.00017)** [low count]</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
@@ -2020,19 +2020,19 @@
           <t>-1.08 (FDR 0.3)</t>
         </is>
       </c>
-      <c r="L15" s="10" t="inlineStr">
-        <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="M15" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="N15" s="10" t="inlineStr">
-        <is>
-          <t>NE</t>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>+4.78 (FDR 0.021)** [low count]</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
+        <is>
+          <t>pass</t>
         </is>
       </c>
       <c r="O15" s="4" t="inlineStr">
@@ -2045,9 +2045,9 @@
           <t>opposite, n.s.</t>
         </is>
       </c>
-      <c r="Q15" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="Q15" s="4" t="inlineStr">
+        <is>
+          <t>+3.94 (FDR 0.0049)** [low count]</t>
         </is>
       </c>
       <c r="R15" s="5" t="inlineStr">
@@ -2057,17 +2057,17 @@
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="T15" s="8" t="inlineStr">
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="T15" s="7" t="inlineStr">
         <is>
           <t>Gao opposite (-1.08)</t>
         </is>
       </c>
-      <c r="U15" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
+      <c r="U15" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2121,7 @@
           <t>-0.01 (FDR 0.98)</t>
         </is>
       </c>
-      <c r="L16" s="9" t="inlineStr">
+      <c r="L16" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2131,7 +2131,7 @@
           <t>+0.46 (FDR 0.094)</t>
         </is>
       </c>
-      <c r="N16" s="9" t="inlineStr">
+      <c r="N16" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2161,7 +2161,7 @@
           <t>H-new2</t>
         </is>
       </c>
-      <c r="T16" s="8" t="inlineStr">
+      <c r="T16" s="7" t="inlineStr">
         <is>
           <t>HGCA opposite (-0.01); Gao opposite (-0.01)</t>
         </is>
@@ -2207,14 +2207,14 @@
           <t>Pikkupeura et al., Science Advances, 2023</t>
         </is>
       </c>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="J17" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>-1.39 (FDR 0.11) [low count]</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>+4.57 (FDR 0.00055)** [low count]</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
@@ -2222,19 +2222,19 @@
           <t>-0.41 (FDR 0.97)</t>
         </is>
       </c>
-      <c r="L17" s="10" t="inlineStr">
-        <is>
-          <t>NE</t>
-        </is>
-      </c>
-      <c r="M17" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="N17" s="10" t="inlineStr">
-        <is>
-          <t>NE</t>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>fail</t>
+        </is>
+      </c>
+      <c r="M17" s="9" t="inlineStr">
+        <is>
+          <t>NA (zero_expression)</t>
+        </is>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>fail</t>
         </is>
       </c>
       <c r="O17" s="4" t="inlineStr">
@@ -2247,9 +2247,9 @@
           <t>concordant</t>
         </is>
       </c>
-      <c r="Q17" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="Q17" s="4" t="inlineStr">
+        <is>
+          <t>-1.52 (FDR 0.00035)* [low count]</t>
         </is>
       </c>
       <c r="R17" s="4" t="inlineStr">
@@ -2259,12 +2259,12 @@
       </c>
       <c r="S17" s="4" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="T17" s="8" t="inlineStr">
-        <is>
-          <t>Gao opposite (-0.41); TCGA bulk significantly tumour-low (-1.03)</t>
+          <t>H-new2</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-1.39); Gao opposite (-0.41); TCGA bulk significantly tumour-low (-1.03)</t>
         </is>
       </c>
       <c r="U17" s="4" t="inlineStr">
@@ -2424,7 +2424,7 @@
           <t>-2.99 (FDR 0.0093)*</t>
         </is>
       </c>
-      <c r="L19" s="9" t="inlineStr">
+      <c r="L19" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2464,7 +2464,7 @@
           <t>H-new2</t>
         </is>
       </c>
-      <c r="T19" s="8" t="inlineStr">
+      <c r="T19" s="7" t="inlineStr">
         <is>
           <t>HGCA opposite (-3.60); Gao opposite (-2.99); GSE44433 significantly adult-high (-4.17)</t>
         </is>
@@ -2565,7 +2565,7 @@
           <t>H-new2</t>
         </is>
       </c>
-      <c r="T20" s="8" t="inlineStr">
+      <c r="T20" s="7" t="inlineStr">
         <is>
           <t>Gao opposite (-1.04); GSE44433 significantly adult-high (-3.02)</t>
         </is>
@@ -2626,7 +2626,7 @@
           <t>-0.84 (FDR 0.61)</t>
         </is>
       </c>
-      <c r="L21" s="9" t="inlineStr">
+      <c r="L21" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2636,7 +2636,7 @@
           <t>-3.26 (FDR 2.6e-09)*</t>
         </is>
       </c>
-      <c r="N21" s="9" t="inlineStr">
+      <c r="N21" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2666,7 +2666,7 @@
           <t>none</t>
         </is>
       </c>
-      <c r="T21" s="8" t="inlineStr">
+      <c r="T21" s="7" t="inlineStr">
         <is>
           <t>HGCA opposite (-3.87); H-new2 opposite (-3.92); Gao opposite (-0.84); GSE44433 significantly adult-high (-0.63)</t>
         </is>
@@ -2727,7 +2727,7 @@
           <t>+0.91 (FDR 0.54)</t>
         </is>
       </c>
-      <c r="L22" s="9" t="inlineStr">
+      <c r="L22" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2742,12 +2742,12 @@
           <t>pass</t>
         </is>
       </c>
-      <c r="O22" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="P22" s="7" t="inlineStr">
+      <c r="O22" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="P22" s="9" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2767,7 +2767,7 @@
           <t>none</t>
         </is>
       </c>
-      <c r="T22" s="8" t="inlineStr">
+      <c r="T22" s="7" t="inlineStr">
         <is>
           <t>H-new2 opposite (-0.24)</t>
         </is>
@@ -2820,7 +2820,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>+3.31 (FDR 0.00099)**</t>
+          <t>+3.31 (FDR 0.001)**</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
@@ -2843,12 +2843,12 @@
           <t>pass</t>
         </is>
       </c>
-      <c r="O23" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="P23" s="7" t="inlineStr">
+      <c r="O23" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="P23" s="9" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2868,7 +2868,7 @@
           <t>H-new2</t>
         </is>
       </c>
-      <c r="T23" s="8" t="inlineStr">
+      <c r="T23" s="7" t="inlineStr">
         <is>
           <t>TCGA bulk significantly tumour-low (-0.46)</t>
         </is>
@@ -2939,7 +2939,7 @@
           <t>+0.01 (FDR 0.98)</t>
         </is>
       </c>
-      <c r="N24" s="9" t="inlineStr">
+      <c r="N24" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -2969,7 +2969,7 @@
           <t>H-new2</t>
         </is>
       </c>
-      <c r="T24" s="8" t="inlineStr">
+      <c r="T24" s="7" t="inlineStr">
         <is>
           <t>Gao opposite (-1.54)</t>
         </is>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>-4.26 (FDR 2.1e-13)*</t>
+          <t>-4.26 (FDR 2.2e-13)*</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
@@ -3030,19 +3030,19 @@
           <t>-0.80 (FDR 0.87)</t>
         </is>
       </c>
-      <c r="L25" s="9" t="inlineStr">
+      <c r="L25" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
       </c>
-      <c r="M25" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="N25" s="10" t="inlineStr">
-        <is>
-          <t>NE</t>
+      <c r="M25" s="4" t="inlineStr">
+        <is>
+          <t>-1.24 (FDR 0.45) [low count]</t>
+        </is>
+      </c>
+      <c r="N25" s="8" t="inlineStr">
+        <is>
+          <t>fail</t>
         </is>
       </c>
       <c r="O25" s="4" t="inlineStr">
@@ -3070,7 +3070,7 @@
           <t>none</t>
         </is>
       </c>
-      <c r="T25" s="8" t="inlineStr">
+      <c r="T25" s="7" t="inlineStr">
         <is>
           <t>HGCA opposite (-5.82); H-new2 opposite (-4.26); Gao opposite (-0.80)</t>
         </is>
@@ -3136,14 +3136,14 @@
           <t>pass</t>
         </is>
       </c>
-      <c r="M26" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="N26" s="10" t="inlineStr">
-        <is>
-          <t>NE</t>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>+7.18 (FDR 0.00076)**</t>
+        </is>
+      </c>
+      <c r="N26" s="6" t="inlineStr">
+        <is>
+          <t>pass</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr">
@@ -3217,19 +3217,19 @@
           <t>Yui et al., Cell Stem Cell, 2018</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="K27" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="J27" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
         </is>
       </c>
       <c r="L27" s="10" t="inlineStr">
@@ -3242,29 +3242,29 @@
           <t>-6.51 (FDR 5.6e-06)*</t>
         </is>
       </c>
-      <c r="N27" s="9" t="inlineStr">
+      <c r="N27" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
       </c>
-      <c r="O27" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="P27" s="7" t="inlineStr">
+      <c r="O27" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="P27" s="9" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="Q27" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="R27" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
+      <c r="Q27" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="R27" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
         </is>
       </c>
       <c r="S27" s="4" t="inlineStr">
@@ -3333,7 +3333,7 @@
           <t>+0.13 (FDR 0.77)</t>
         </is>
       </c>
-      <c r="L28" s="9" t="inlineStr">
+      <c r="L28" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3373,7 +3373,7 @@
           <t>none</t>
         </is>
       </c>
-      <c r="T28" s="8" t="inlineStr">
+      <c r="T28" s="7" t="inlineStr">
         <is>
           <t>HGCA opposite (-5.05); GSE44433 significantly adult-high (-2.37); TCGA bulk significantly tumour-low (-1.75)</t>
         </is>
@@ -3444,7 +3444,7 @@
           <t>-0.07 (FDR 0.63)</t>
         </is>
       </c>
-      <c r="N29" s="9" t="inlineStr">
+      <c r="N29" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3474,7 +3474,7 @@
           <t>H-new2</t>
         </is>
       </c>
-      <c r="T29" s="8" t="inlineStr">
+      <c r="T29" s="7" t="inlineStr">
         <is>
           <t>HGCA opposite (-1.07)</t>
         </is>
@@ -3520,14 +3520,14 @@
           <t>Buissant des Amorie et al., Nature, 2026</t>
         </is>
       </c>
-      <c r="I30" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="J30" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>-4.57 (FDR 2.3e-05)* [low count]</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>+0.40 (FDR 0.76) [low count]</t>
         </is>
       </c>
       <c r="K30" s="4" t="inlineStr">
@@ -3535,9 +3535,9 @@
           <t>+0.12 (FDR 0.97)</t>
         </is>
       </c>
-      <c r="L30" s="10" t="inlineStr">
-        <is>
-          <t>NE</t>
+      <c r="L30" s="8" t="inlineStr">
+        <is>
+          <t>fail</t>
         </is>
       </c>
       <c r="M30" s="4" t="inlineStr">
@@ -3545,7 +3545,7 @@
           <t>-2.83 (FDR 1.6e-05)*</t>
         </is>
       </c>
-      <c r="N30" s="9" t="inlineStr">
+      <c r="N30" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3575,9 +3575,9 @@
           <t>none</t>
         </is>
       </c>
-      <c r="T30" s="8" t="inlineStr">
-        <is>
-          <t>GSE44433 significantly adult-high (-1.09)</t>
+      <c r="T30" s="7" t="inlineStr">
+        <is>
+          <t>HGCA opposite (-4.57); GSE44433 significantly adult-high (-1.09)</t>
         </is>
       </c>
       <c r="U30" s="4" t="inlineStr">
@@ -3621,14 +3621,14 @@
           <t>Ganesh et al., Nature Cancer, 2020 | Ganesh et al., Nature Cancer, 2020; Moorman et al., Nature, 2025</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>+1.98 (FDR 0.0036)**</t>
-        </is>
-      </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>+1.98 (FDR 0.0036)** [low count]</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>+5.76 (FDR 9.2e-05)** [low count]</t>
         </is>
       </c>
       <c r="K31" s="4" t="inlineStr">
@@ -3646,7 +3646,7 @@
           <t>-4.97 (FDR 8.1e-10)*</t>
         </is>
       </c>
-      <c r="N31" s="9" t="inlineStr">
+      <c r="N31" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3661,9 +3661,9 @@
           <t>significant contradiction</t>
         </is>
       </c>
-      <c r="Q31" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="Q31" s="5" t="inlineStr">
+        <is>
+          <t>+7.89 (FDR 2.7e-05)**</t>
         </is>
       </c>
       <c r="R31" s="4" t="inlineStr">
@@ -3673,10 +3673,10 @@
       </c>
       <c r="S31" s="4" t="inlineStr">
         <is>
-          <t>HGCA</t>
-        </is>
-      </c>
-      <c r="T31" s="8" t="inlineStr">
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="T31" s="7" t="inlineStr">
         <is>
           <t>GSE44433 significantly adult-high (-3.76); TCGA bulk significantly tumour-low (-1.27)</t>
         </is>
@@ -3737,7 +3737,7 @@
           <t>-1.75 (FDR 0.26)</t>
         </is>
       </c>
-      <c r="L32" s="9" t="inlineStr">
+      <c r="L32" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
@@ -3747,17 +3747,17 @@
           <t>+0.05 (FDR 0.89)</t>
         </is>
       </c>
-      <c r="N32" s="9" t="inlineStr">
+      <c r="N32" s="8" t="inlineStr">
         <is>
           <t>fail</t>
         </is>
       </c>
-      <c r="O32" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="P32" s="7" t="inlineStr">
+      <c r="O32" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="P32" s="9" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -3777,7 +3777,7 @@
           <t>none</t>
         </is>
       </c>
-      <c r="T32" s="8" t="inlineStr">
+      <c r="T32" s="7" t="inlineStr">
         <is>
           <t>HGCA opposite (-2.68); H-new2 opposite (-0.30); Gao opposite (-1.75)</t>
         </is>
@@ -3906,9 +3906,9 @@
           <t>+9.46 (FDR 4.4e-15)**</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -4076,34 +4076,34 @@
           <t>LY6A</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
         </is>
       </c>
     </row>
@@ -4150,34 +4150,34 @@
           <t>SPRR1A</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
         </is>
       </c>
     </row>
@@ -4350,14 +4350,14 @@
           <t>+14.48 (FDR 9.5e-16)**</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -4409,9 +4409,9 @@
           <t>SOX17</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -4424,9 +4424,9 @@
           <t>+11.16 (FDR 3.1e-11)**</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -4599,14 +4599,14 @@
           <t>+0.12 (FDR 0.46)</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -4779,34 +4779,34 @@
           <t>REG3B</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>NA (no one2one orthologue)</t>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>NA (no_1to1_orthologue)</t>
         </is>
       </c>
     </row>
@@ -4890,9 +4890,9 @@
           <t>MMP7</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -4927,9 +4927,9 @@
           <t>L1CAM</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -4942,9 +4942,9 @@
           <t>-1.56 (FDR 7.7e-10)*</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>NA (supportive dataset; absent or filtered, not re-audited)</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -5006,7 +5006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5214,9 +5214,9 @@
           <t>concordant</t>
         </is>
       </c>
-      <c r="Q2" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="Q2" s="4" t="inlineStr">
+        <is>
+          <t>+3.89 (FDR 9.3e-06)** [low count]</t>
         </is>
       </c>
       <c r="R2" s="4" t="inlineStr">
@@ -5229,7 +5229,7 @@
           <t>HGCA, H-new2</t>
         </is>
       </c>
-      <c r="T2" s="8" t="inlineStr">
+      <c r="T2" s="7" t="inlineStr">
         <is>
           <t>Gao opposite (-0.16)</t>
         </is>
@@ -5330,7 +5330,7 @@
           <t>HGCA, H-new2</t>
         </is>
       </c>
-      <c r="T3" s="8" t="inlineStr">
+      <c r="T3" s="7" t="inlineStr">
         <is>
           <t>TCGA bulk significantly tumour-low (-2.31)</t>
         </is>
@@ -5431,7 +5431,7 @@
           <t>HGCA, H-new2</t>
         </is>
       </c>
-      <c r="T4" s="8" t="inlineStr">
+      <c r="T4" s="7" t="inlineStr">
         <is>
           <t>TCGA bulk significantly tumour-low (-0.33)</t>
         </is>
@@ -5482,9 +5482,9 @@
           <t>+2.52 (FDR 0.029)**</t>
         </is>
       </c>
-      <c r="J5" s="7" t="inlineStr">
-        <is>
-          <t>NA (not measured)</t>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>+7.30 (FDR 0.0021)**</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -5492,9 +5492,9 @@
           <t>-0.01 (FDR 0.83)</t>
         </is>
       </c>
-      <c r="L5" s="9" t="inlineStr">
-        <is>
-          <t>fail</t>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>pass</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
@@ -5529,10 +5529,10 @@
       </c>
       <c r="S5" s="4" t="inlineStr">
         <is>
-          <t>HGCA</t>
-        </is>
-      </c>
-      <c r="T5" s="8" t="inlineStr">
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="T5" s="7" t="inlineStr">
         <is>
           <t>Gao opposite (-0.01)</t>
         </is>
@@ -5546,99 +5546,200 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
+          <t>ANKRD1</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>ANKRD1</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Pikkupeura et al., Science Advances, 2023 | Hartl et al., Sci Adv, 2024; Yui et al., Cell Stem Cell, 2018</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>+5.63 (FDR 0.003)** [low count]</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>+4.46 (FDR 0.00017)** [low count]</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>-1.08 (FDR 0.3)</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>+4.78 (FDR 0.021)** [low count]</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>-0.02 (FDR 0.83)</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>opposite, n.s.</t>
+        </is>
+      </c>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>+3.94 (FDR 0.0049)** [low count]</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
+        <is>
+          <t>+2.49 (FDR 9.9e-08)**</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>HGCA, H-new2</t>
+        </is>
+      </c>
+      <c r="T6" s="7" t="inlineStr">
+        <is>
+          <t>Gao opposite (-1.08)</t>
+        </is>
+      </c>
+      <c r="U6" s="6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
           <t>RBP1</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>RBP1</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>provenance unresolved</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>none identified</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>+5.54 (FDR 1.8e-05)**</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>+1.43 (FDR 0.13)</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>+4.24 (FDR 0.024)**</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>+2.88 (FDR 8.5e-06)**</t>
         </is>
       </c>
-      <c r="N6" s="6" t="inlineStr">
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O7" s="5" t="inlineStr">
         <is>
           <t>+2.84 (FDR 6.9e-09)**</t>
         </is>
       </c>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>concordant</t>
         </is>
       </c>
-      <c r="Q6" s="5" t="inlineStr">
+      <c r="Q7" s="5" t="inlineStr">
         <is>
           <t>+6.31 (FDR 3e-11)**</t>
         </is>
       </c>
-      <c r="R6" s="5" t="inlineStr">
+      <c r="R7" s="5" t="inlineStr">
         <is>
           <t>+1.57 (FDR 7e-07)**</t>
         </is>
       </c>
-      <c r="S6" s="4" t="inlineStr">
+      <c r="S7" s="4" t="inlineStr">
         <is>
           <t>HGCA, Gao</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr">
+      <c r="T7" s="4" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="U6" s="6" t="inlineStr">
+      <c r="U7" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
@@ -10551,13 +10652,13 @@
         </is>
       </c>
       <c r="D2" s="4" t="n">
-        <v>0.19798865128589</v>
+        <v>0.198091194516698</v>
       </c>
       <c r="E2" s="4" t="n">
-        <v>0.749220062902486</v>
+        <v>0.749116984562208</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>0.800474915981509</v>
+        <v>0.800400507654875</v>
       </c>
       <c r="G2" s="4" t="b">
         <v>1</v>
@@ -10583,13 +10684,13 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>4.08526804610829</v>
+        <v>4.08514588812678</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>4.03296851332847e-06</v>
+        <v>4.03985721287775e-06</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>1.82819733762252e-05</v>
+        <v>1.83261385272533e-05</v>
       </c>
       <c r="G3" s="4" t="b">
         <v>1</v>
@@ -10647,13 +10748,13 @@
         </is>
       </c>
       <c r="D5" s="4" t="n">
-        <v>7.78164418621455</v>
+        <v>7.78169550419528</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>0.0005418655447418001</v>
+        <v>0.000534045827929</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0.0016665275728096</v>
+        <v>0.001644490713609</v>
       </c>
       <c r="G5" s="4" t="b">
         <v>1</v>
@@ -10711,13 +10812,13 @@
         </is>
       </c>
       <c r="D7" s="4" t="n">
-        <v>4.25904379124654</v>
+        <v>4.25895064102979</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>7.182211571553239e-12</v>
+        <v>7.178488696309739e-12</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>3.76963504484094e-11</v>
+        <v>3.76896294015891e-11</v>
       </c>
       <c r="G7" s="4" t="b">
         <v>1</v>
@@ -10959,13 +11060,13 @@
         </is>
       </c>
       <c r="D15" s="4" t="n">
-        <v>6.05432625132332</v>
+        <v>6.0544899983769</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>1.33898947629916e-09</v>
+        <v>1.33415092504576e-09</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>6.49574077276029e-08</v>
+        <v>6.48912066993597e-08</v>
       </c>
       <c r="G15" s="4" t="b">
         <v>1</v>
@@ -10991,13 +11092,13 @@
         </is>
       </c>
       <c r="D16" s="4" t="n">
-        <v>2.77075537774903</v>
+        <v>2.77086011208077</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.0061981986054554</v>
+        <v>0.0062039391991986</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0.0121391902825689</v>
+        <v>0.0121489398677049</v>
       </c>
       <c r="G16" s="4" t="b">
         <v>1</v>
@@ -11055,13 +11156,13 @@
         </is>
       </c>
       <c r="D18" s="4" t="n">
-        <v>8.29188190022181</v>
+        <v>8.29201409995539</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>1.44179212394248e-10</v>
+        <v>1.4434282967628e-10</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>7.21329989010664e-09</v>
+        <v>7.194512329449432e-09</v>
       </c>
       <c r="G18" s="4" t="b">
         <v>1</v>
@@ -11118,14 +11219,20 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
+      <c r="D20" s="4" t="n">
+        <v>3.89444791114916</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>3.84795124228494e-06</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>9.330155238797769e-06</v>
+      </c>
       <c r="G20" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H20" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -11355,13 +11462,13 @@
         </is>
       </c>
       <c r="D28" s="4" t="n">
-        <v>-2.37689523735549</v>
+        <v>-2.37669617413341</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>1.77035136356332e-06</v>
+        <v>1.76994742285677e-06</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>1.6964120385835e-05</v>
+        <v>1.69570708828034e-05</v>
       </c>
       <c r="G28" s="4" t="b">
         <v>1</v>
@@ -11387,13 +11494,13 @@
         </is>
       </c>
       <c r="D29" s="4" t="n">
-        <v>-0.931228468737944</v>
+        <v>-0.9310513705812899</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>0.180218025785427</v>
+        <v>0.180380120361163</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>0.239594547741475</v>
+        <v>0.239799643213807</v>
       </c>
       <c r="G29" s="4" t="b">
         <v>1</v>
@@ -11451,13 +11558,13 @@
         </is>
       </c>
       <c r="D31" s="4" t="n">
-        <v>9.68991510142647</v>
+        <v>9.68996588228379</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>1.43970264426793e-06</v>
+        <v>1.4354159599431e-06</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>1.1060704561906e-05</v>
+        <v>1.10374536688927e-05</v>
       </c>
       <c r="G31" s="4" t="b">
         <v>1</v>
@@ -11515,13 +11622,13 @@
         </is>
       </c>
       <c r="D33" s="4" t="n">
-        <v>2.84220968978987</v>
+        <v>2.84217173214838</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>1.17188992894437e-12</v>
+        <v>1.17140136878295e-12</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>6.82874480403112e-12</v>
+        <v>6.82822027060991e-12</v>
       </c>
       <c r="G33" s="4" t="b">
         <v>1</v>
@@ -11763,13 +11870,13 @@
         </is>
       </c>
       <c r="D41" s="4" t="n">
-        <v>2.39020429652892</v>
+        <v>2.39037482841822</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0.0011297535325881</v>
+        <v>0.0011288682249231</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0.0033384451276678</v>
+        <v>0.0033354712708529</v>
       </c>
       <c r="G41" s="4" t="b">
         <v>1</v>
@@ -11795,13 +11902,13 @@
         </is>
       </c>
       <c r="D42" s="4" t="n">
-        <v>2.34510833736241</v>
+        <v>2.3450942374854</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>1.89352078133194e-05</v>
+        <v>1.89352471298127e-05</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>7.133106575596e-05</v>
+        <v>7.13959785637618e-05</v>
       </c>
       <c r="G42" s="4" t="b">
         <v>1</v>
@@ -11859,13 +11966,13 @@
         </is>
       </c>
       <c r="D44" s="4" t="n">
-        <v>5.2397749056071</v>
+        <v>5.2399202234077</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>5.805924394285639e-11</v>
+        <v>5.780357218184769e-11</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>3.82673650423361e-09</v>
+        <v>3.81102957583093e-09</v>
       </c>
       <c r="G44" s="4" t="b">
         <v>1</v>
@@ -11923,13 +12030,13 @@
         </is>
       </c>
       <c r="D46" s="4" t="n">
-        <v>1.49510505291086</v>
+        <v>1.49507163709415</v>
       </c>
       <c r="E46" s="4" t="n">
-        <v>1.96773871980725e-06</v>
+        <v>1.96700225462924e-06</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>4.95593628556767e-06</v>
+        <v>4.95661641160515e-06</v>
       </c>
       <c r="G46" s="4" t="b">
         <v>1</v>
@@ -12171,13 +12278,13 @@
         </is>
       </c>
       <c r="D54" s="4" t="n">
-        <v>1.98732901132584</v>
+        <v>1.98746925258846</v>
       </c>
       <c r="E54" s="4" t="n">
-        <v>6.7248354618785e-09</v>
+        <v>6.7153322758486e-09</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>2.23792468342588e-07</v>
+        <v>2.23109397702074e-07</v>
       </c>
       <c r="G54" s="4" t="b">
         <v>1</v>
@@ -12203,13 +12310,13 @@
         </is>
       </c>
       <c r="D55" s="4" t="n">
-        <v>1.76569125688894</v>
+        <v>1.76568340553857</v>
       </c>
       <c r="E55" s="4" t="n">
-        <v>0.0013225792046715</v>
+        <v>0.0013239528305751</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>0.0030586054052522</v>
+        <v>0.0030611151762252</v>
       </c>
       <c r="G55" s="4" t="b">
         <v>1</v>
@@ -12267,13 +12374,13 @@
         </is>
       </c>
       <c r="D57" s="4" t="n">
-        <v>-1.22430801559859</v>
+        <v>-1.22416301109396</v>
       </c>
       <c r="E57" s="4" t="n">
-        <v>0.0062117530272515</v>
+        <v>0.006218158071233</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>0.0136881641106156</v>
+        <v>0.0137017586354537</v>
       </c>
       <c r="G57" s="4" t="b">
         <v>1</v>
@@ -12331,13 +12438,13 @@
         </is>
       </c>
       <c r="D59" s="4" t="n">
-        <v>1.65228981386363</v>
+        <v>1.65227949664548</v>
       </c>
       <c r="E59" s="4" t="n">
-        <v>3.14204380887234e-18</v>
+        <v>3.13845534990033e-18</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>4.53590135709114e-17</v>
+        <v>4.53226248515568e-17</v>
       </c>
       <c r="G59" s="4" t="b">
         <v>1</v>
@@ -12579,13 +12686,13 @@
         </is>
       </c>
       <c r="D67" s="4" t="n">
-        <v>2.41044937648594</v>
+        <v>2.41063120397189</v>
       </c>
       <c r="E67" s="4" t="n">
-        <v>6.09503618318197e-06</v>
+        <v>6.08357602849857e-06</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>4.52338575262075e-05</v>
+        <v>4.51260452275789e-05</v>
       </c>
       <c r="G67" s="4" t="b">
         <v>1</v>
@@ -12611,13 +12718,13 @@
         </is>
       </c>
       <c r="D68" s="4" t="n">
-        <v>2.50419699416761</v>
+        <v>2.50428974813114</v>
       </c>
       <c r="E68" s="4" t="n">
-        <v>0.0001056220241727</v>
+        <v>0.0001058772544516</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>0.0003250612605267</v>
+        <v>0.0003258433655979</v>
       </c>
       <c r="G68" s="4" t="b">
         <v>1</v>
@@ -12675,13 +12782,13 @@
         </is>
       </c>
       <c r="D70" s="4" t="n">
-        <v>2.94613516104027</v>
+        <v>2.94629066427778</v>
       </c>
       <c r="E70" s="4" t="n">
-        <v>4.38131580064081e-08</v>
+        <v>4.37147897207499e-08</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>6.21749815462695e-07</v>
+        <v>6.20593482793803e-07</v>
       </c>
       <c r="G70" s="4" t="b">
         <v>1</v>
@@ -12739,13 +12846,13 @@
         </is>
       </c>
       <c r="D72" s="4" t="n">
-        <v>2.95811168926125</v>
+        <v>2.95805174857796</v>
       </c>
       <c r="E72" s="4" t="n">
-        <v>9.498025206415731e-15</v>
+        <v>9.470639044637812e-15</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>7.4843420071574e-14</v>
+        <v>7.465301050682061e-14</v>
       </c>
       <c r="G72" s="4" t="b">
         <v>1</v>
@@ -13064,9 +13171,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D83" s="4" t="n"/>
-      <c r="E83" s="4" t="n"/>
-      <c r="F83" s="4" t="n"/>
+      <c r="D83" s="4" t="n">
+        <v>-2.26233477967598</v>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>0.0045930375423618</v>
+      </c>
+      <c r="F83" s="4" t="n">
+        <v>0.0105193592414746</v>
+      </c>
       <c r="G83" s="4" t="b">
         <v>1</v>
       </c>
@@ -13325,13 +13438,13 @@
         </is>
       </c>
       <c r="D93" s="4" t="n">
-        <v>2.51852984972419</v>
+        <v>2.51871529159197</v>
       </c>
       <c r="E93" s="4" t="n">
-        <v>0.0144161597019829</v>
+        <v>0.0144021515951647</v>
       </c>
       <c r="F93" s="4" t="n">
-        <v>0.0289201264700338</v>
+        <v>0.0288919134399789</v>
       </c>
       <c r="G93" s="4" t="b">
         <v>1</v>
@@ -13356,14 +13469,20 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D94" s="4" t="n"/>
-      <c r="E94" s="4" t="n"/>
-      <c r="F94" s="4" t="n"/>
+      <c r="D94" s="4" t="n">
+        <v>7.29707655873438</v>
+      </c>
+      <c r="E94" s="4" t="n">
+        <v>0.0008739402210126</v>
+      </c>
+      <c r="F94" s="4" t="n">
+        <v>0.0021222636877455</v>
+      </c>
       <c r="G94" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H94" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95">
@@ -13415,13 +13534,13 @@
         </is>
       </c>
       <c r="D96" s="4" t="n">
-        <v>10.0513997206468</v>
+        <v>10.0515380602187</v>
       </c>
       <c r="E96" s="4" t="n">
-        <v>5.53659139386556e-14</v>
+        <v>5.54987135205716e-14</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>2.635465732107369e-11</v>
+        <v>2.63975666666776e-11</v>
       </c>
       <c r="G96" s="4" t="b">
         <v>1</v>
@@ -13479,13 +13598,13 @@
         </is>
       </c>
       <c r="D98" s="4" t="n">
-        <v>6.12870673194068</v>
+        <v>6.12849610079981</v>
       </c>
       <c r="E98" s="4" t="n">
-        <v>3.861565125239149e-18</v>
+        <v>3.85209191803483e-18</v>
       </c>
       <c r="F98" s="4" t="n">
-        <v>5.47771298197193e-17</v>
+        <v>5.46090677791997e-17</v>
       </c>
       <c r="G98" s="4" t="b">
         <v>1</v>
@@ -13726,9 +13845,15 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D106" s="4" t="n"/>
-      <c r="E106" s="4" t="n"/>
-      <c r="F106" s="4" t="n"/>
+      <c r="D106" s="4" t="n">
+        <v>-1.42847347210584</v>
+      </c>
+      <c r="E106" s="4" t="n">
+        <v>0.302991742189323</v>
+      </c>
+      <c r="F106" s="4" t="n">
+        <v>0.384499176577172</v>
+      </c>
       <c r="G106" s="4" t="b">
         <v>1</v>
       </c>
@@ -13862,14 +13987,20 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D111" s="4" t="n"/>
-      <c r="E111" s="4" t="n"/>
-      <c r="F111" s="4" t="n"/>
+      <c r="D111" s="4" t="n">
+        <v>5.08048249168194</v>
+      </c>
+      <c r="E111" s="4" t="n">
+        <v>0.0026634155954816</v>
+      </c>
+      <c r="F111" s="4" t="n">
+        <v>0.0044167933072956</v>
+      </c>
       <c r="G111" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H111" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -14077,13 +14208,13 @@
         </is>
       </c>
       <c r="D119" s="4" t="n">
-        <v>-2.49412446880068</v>
+        <v>-2.49407764042705</v>
       </c>
       <c r="E119" s="4" t="n">
-        <v>0.0013300804174449</v>
+        <v>0.0013283913646226</v>
       </c>
       <c r="F119" s="4" t="n">
-        <v>0.0038312169150928</v>
+        <v>0.0038265922713038</v>
       </c>
       <c r="G119" s="4" t="b">
         <v>1</v>
@@ -14108,14 +14239,20 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D120" s="4" t="n"/>
-      <c r="E120" s="4" t="n"/>
-      <c r="F120" s="4" t="n"/>
+      <c r="D120" s="4" t="n">
+        <v>1.21816780357903</v>
+      </c>
+      <c r="E120" s="4" t="n">
+        <v>0.0293313215006038</v>
+      </c>
+      <c r="F120" s="4" t="n">
+        <v>0.0488364375392265</v>
+      </c>
       <c r="G120" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H120" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121">
@@ -14167,13 +14304,13 @@
         </is>
       </c>
       <c r="D122" s="4" t="n">
-        <v>-0.942039269293886</v>
+        <v>-0.941891336449691</v>
       </c>
       <c r="E122" s="4" t="n">
-        <v>0.0340607584218804</v>
+        <v>0.0341447065640873</v>
       </c>
       <c r="F122" s="4" t="n">
-        <v>0.059984780109645</v>
+        <v>0.0601140192570496</v>
       </c>
       <c r="G122" s="4" t="b">
         <v>1</v>
@@ -14231,13 +14368,13 @@
         </is>
       </c>
       <c r="D124" s="4" t="n">
-        <v>4.55190891741079</v>
+        <v>4.55208861460633</v>
       </c>
       <c r="E124" s="4" t="n">
-        <v>3.26690738255902e-17</v>
+        <v>3.25680070049135e-17</v>
       </c>
       <c r="F124" s="4" t="n">
-        <v>3.90964746694522e-16</v>
+        <v>3.89887842816966e-16</v>
       </c>
       <c r="G124" s="4" t="b">
         <v>1</v>
@@ -14479,13 +14616,13 @@
         </is>
       </c>
       <c r="D132" s="4" t="n">
-        <v>0.954081325459462</v>
+        <v>0.954251293055386</v>
       </c>
       <c r="E132" s="4" t="n">
-        <v>0.0423802441365801</v>
+        <v>0.0423353705842584</v>
       </c>
       <c r="F132" s="4" t="n">
-        <v>0.07262154635300019</v>
+        <v>0.0725609508531735</v>
       </c>
       <c r="G132" s="4" t="b">
         <v>1</v>
@@ -14511,13 +14648,13 @@
         </is>
       </c>
       <c r="D133" s="4" t="n">
-        <v>-1.07750080237949</v>
+        <v>-1.07749105082408</v>
       </c>
       <c r="E133" s="4" t="n">
-        <v>0.009031611015030401</v>
+        <v>0.009036164483080301</v>
       </c>
       <c r="F133" s="4" t="n">
-        <v>0.0170244497823767</v>
+        <v>0.017033426921991</v>
       </c>
       <c r="G133" s="4" t="b">
         <v>1</v>
@@ -14569,13 +14706,13 @@
         </is>
       </c>
       <c r="D135" s="4" t="n">
-        <v>1.03400523977176</v>
+        <v>1.03417377912902</v>
       </c>
       <c r="E135" s="4" t="n">
-        <v>0.0001913431545588</v>
+        <v>0.000188279781741</v>
       </c>
       <c r="F135" s="4" t="n">
-        <v>0.0006752034878866</v>
+        <v>0.0006660053474707</v>
       </c>
       <c r="G135" s="4" t="b">
         <v>1</v>
@@ -14627,13 +14764,13 @@
         </is>
       </c>
       <c r="D137" s="4" t="n">
-        <v>1.34994899681148</v>
+        <v>1.3499503622219</v>
       </c>
       <c r="E137" s="4" t="n">
-        <v>3.55649118340587e-07</v>
+        <v>3.55514715090145e-07</v>
       </c>
       <c r="F137" s="4" t="n">
-        <v>9.80972117705192e-07</v>
+        <v>9.80935027503795e-07</v>
       </c>
       <c r="G137" s="4" t="b">
         <v>1</v>
@@ -14875,13 +15012,13 @@
         </is>
       </c>
       <c r="D145" s="4" t="n">
-        <v>0.382628097563692</v>
+        <v>0.382853420066617</v>
       </c>
       <c r="E145" s="4" t="n">
-        <v>0.473103960554125</v>
+        <v>0.472842263527965</v>
       </c>
       <c r="F145" s="4" t="n">
-        <v>0.554081233634103</v>
+        <v>0.5538262976128649</v>
       </c>
       <c r="G145" s="4" t="b">
         <v>1</v>
@@ -14907,13 +15044,13 @@
         </is>
       </c>
       <c r="D146" s="4" t="n">
-        <v>6.36969425628561</v>
+        <v>6.36968011753382</v>
       </c>
       <c r="E146" s="4" t="n">
-        <v>1.02849644899664e-06</v>
+        <v>1.0296524813322e-06</v>
       </c>
       <c r="F146" s="4" t="n">
-        <v>5.64348640188959e-06</v>
+        <v>5.65210265690817e-06</v>
       </c>
       <c r="G146" s="4" t="b">
         <v>1</v>
@@ -14971,13 +15108,13 @@
         </is>
       </c>
       <c r="D148" s="4" t="n">
-        <v>4.71853596181636</v>
+        <v>4.71868634753493</v>
       </c>
       <c r="E148" s="4" t="n">
-        <v>1.05599860213055e-08</v>
+        <v>1.05278927967348e-08</v>
       </c>
       <c r="F148" s="4" t="n">
-        <v>1.95815673938247e-07</v>
+        <v>1.95279214856426e-07</v>
       </c>
       <c r="G148" s="4" t="b">
         <v>1</v>
@@ -15035,13 +15172,13 @@
         </is>
       </c>
       <c r="D150" s="4" t="n">
-        <v>0.628181546646409</v>
+        <v>0.628200726748787</v>
       </c>
       <c r="E150" s="4" t="n">
-        <v>0.0182260506391194</v>
+        <v>0.0182230735847301</v>
       </c>
       <c r="F150" s="4" t="n">
-        <v>0.0265645185155706</v>
+        <v>0.0265560472610148</v>
       </c>
       <c r="G150" s="4" t="b">
         <v>1</v>
@@ -15283,13 +15420,13 @@
         </is>
       </c>
       <c r="D158" s="4" t="n">
-        <v>-0.361591332412759</v>
+        <v>-0.361475057053875</v>
       </c>
       <c r="E158" s="4" t="n">
-        <v>0.604854294765779</v>
+        <v>0.604971930912678</v>
       </c>
       <c r="F158" s="4" t="n">
-        <v>0.676263869882563</v>
+        <v>0.676334995649003</v>
       </c>
       <c r="G158" s="4" t="b">
         <v>1</v>
@@ -15315,13 +15452,13 @@
         </is>
       </c>
       <c r="D159" s="4" t="n">
-        <v>7.35140825550013</v>
+        <v>7.35140433689018</v>
       </c>
       <c r="E159" s="4" t="n">
-        <v>1.62741979236739e-14</v>
+        <v>1.62930106407932e-14</v>
       </c>
       <c r="F159" s="4" t="n">
-        <v>9.866397879417609e-13</v>
+        <v>9.881777185391641e-13</v>
       </c>
       <c r="G159" s="4" t="b">
         <v>1</v>
@@ -15379,13 +15516,13 @@
         </is>
       </c>
       <c r="D161" s="4" t="n">
-        <v>1.50891123127904</v>
+        <v>1.50904347834348</v>
       </c>
       <c r="E161" s="4" t="n">
-        <v>0.0148659599062637</v>
+        <v>0.0148719347385706</v>
       </c>
       <c r="F161" s="4" t="n">
-        <v>0.0293005758981488</v>
+        <v>0.0293124799242687</v>
       </c>
       <c r="G161" s="4" t="b">
         <v>1</v>
@@ -15437,13 +15574,13 @@
         </is>
       </c>
       <c r="D163" s="4" t="n">
-        <v>1.01939227713914</v>
+        <v>1.01947519585084</v>
       </c>
       <c r="E163" s="4" t="n">
-        <v>0.0004851373297352</v>
+        <v>0.0004843600084661</v>
       </c>
       <c r="F163" s="4" t="n">
-        <v>0.0008941031098306</v>
+        <v>0.0008926383959459001</v>
       </c>
       <c r="G163" s="4" t="b">
         <v>1</v>
@@ -15684,14 +15821,20 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D171" s="4" t="n"/>
-      <c r="E171" s="4" t="n"/>
-      <c r="F171" s="4" t="n"/>
+      <c r="D171" s="4" t="n">
+        <v>5.63115492026782</v>
+      </c>
+      <c r="E171" s="4" t="n">
+        <v>0.0009964186530590001</v>
+      </c>
+      <c r="F171" s="4" t="n">
+        <v>0.0030063065983092</v>
+      </c>
       <c r="G171" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H171" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172">
@@ -15710,14 +15853,20 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D172" s="4" t="n"/>
-      <c r="E172" s="4" t="n"/>
-      <c r="F172" s="4" t="n"/>
+      <c r="D172" s="4" t="n">
+        <v>4.45501086320865</v>
+      </c>
+      <c r="E172" s="4" t="n">
+        <v>5.06566696251194e-05</v>
+      </c>
+      <c r="F172" s="4" t="n">
+        <v>0.000169461325293</v>
+      </c>
       <c r="G172" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H172" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="173">
@@ -15768,14 +15917,20 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D174" s="4" t="n"/>
-      <c r="E174" s="4" t="n"/>
-      <c r="F174" s="4" t="n"/>
+      <c r="D174" s="4" t="n">
+        <v>4.77529874241249</v>
+      </c>
+      <c r="E174" s="4" t="n">
+        <v>0.0103058136889312</v>
+      </c>
+      <c r="F174" s="4" t="n">
+        <v>0.0211777236088854</v>
+      </c>
       <c r="G174" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H174" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175">
@@ -15826,14 +15981,20 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D176" s="4" t="n"/>
-      <c r="E176" s="4" t="n"/>
-      <c r="F176" s="4" t="n"/>
+      <c r="D176" s="4" t="n">
+        <v>3.93612535126544</v>
+      </c>
+      <c r="E176" s="4" t="n">
+        <v>0.0029543397400189</v>
+      </c>
+      <c r="F176" s="4" t="n">
+        <v>0.0048646671727171</v>
+      </c>
       <c r="G176" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H176" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="177">
@@ -16059,13 +16220,13 @@
         </is>
       </c>
       <c r="D184" s="4" t="n">
-        <v>-0.0079116097550831</v>
+        <v>-0.0075781693211536</v>
       </c>
       <c r="E184" s="4" t="n">
-        <v>0.988473049419114</v>
+        <v>0.988957792780522</v>
       </c>
       <c r="F184" s="4" t="n">
-        <v>0.991921018217986</v>
+        <v>0.992077533451754</v>
       </c>
       <c r="G184" s="4" t="b">
         <v>1</v>
@@ -16091,13 +16252,13 @@
         </is>
       </c>
       <c r="D185" s="4" t="n">
-        <v>1.93596804565604</v>
+        <v>1.93595786799713</v>
       </c>
       <c r="E185" s="4" t="n">
-        <v>1.94296808530943e-06</v>
+        <v>1.94502658668101e-06</v>
       </c>
       <c r="F185" s="4" t="n">
-        <v>9.67203805884672e-06</v>
+        <v>9.69265085947919e-06</v>
       </c>
       <c r="G185" s="4" t="b">
         <v>1</v>
@@ -16155,13 +16316,13 @@
         </is>
       </c>
       <c r="D187" s="4" t="n">
-        <v>0.456557736669998</v>
+        <v>0.456710333954212</v>
       </c>
       <c r="E187" s="4" t="n">
-        <v>0.0575847323533967</v>
+        <v>0.0575153846421442</v>
       </c>
       <c r="F187" s="4" t="n">
-        <v>0.09429136964126481</v>
+        <v>0.09421769897467119</v>
       </c>
       <c r="G187" s="4" t="b">
         <v>1</v>
@@ -16219,13 +16380,13 @@
         </is>
       </c>
       <c r="D189" s="4" t="n">
-        <v>2.68701270314905</v>
+        <v>2.68701601674666</v>
       </c>
       <c r="E189" s="4" t="n">
-        <v>1.48745023055985e-22</v>
+        <v>1.48548009770411e-22</v>
       </c>
       <c r="F189" s="4" t="n">
-        <v>4.660888824799061e-21</v>
+        <v>4.65629912928532e-21</v>
       </c>
       <c r="G189" s="4" t="b">
         <v>1</v>
@@ -16466,9 +16627,15 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D197" s="4" t="n"/>
-      <c r="E197" s="4" t="n"/>
-      <c r="F197" s="4" t="n"/>
+      <c r="D197" s="4" t="n">
+        <v>-1.38526280278438</v>
+      </c>
+      <c r="E197" s="4" t="n">
+        <v>0.0696923106312682</v>
+      </c>
+      <c r="F197" s="4" t="n">
+        <v>0.111148188045999</v>
+      </c>
       <c r="G197" s="4" t="b">
         <v>1</v>
       </c>
@@ -16492,14 +16659,20 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D198" s="4" t="n"/>
-      <c r="E198" s="4" t="n"/>
-      <c r="F198" s="4" t="n"/>
+      <c r="D198" s="4" t="n">
+        <v>4.57018179993649</v>
+      </c>
+      <c r="E198" s="4" t="n">
+        <v>0.0001920851528004</v>
+      </c>
+      <c r="F198" s="4" t="n">
+        <v>0.000553371399842</v>
+      </c>
       <c r="G198" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H198" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="199">
@@ -16608,9 +16781,15 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D202" s="4" t="n"/>
-      <c r="E202" s="4" t="n"/>
-      <c r="F202" s="4" t="n"/>
+      <c r="D202" s="4" t="n">
+        <v>-1.51940843748415</v>
+      </c>
+      <c r="E202" s="4" t="n">
+        <v>0.0001811039182849</v>
+      </c>
+      <c r="F202" s="4" t="n">
+        <v>0.0003534327230461</v>
+      </c>
       <c r="G202" s="4" t="b">
         <v>1</v>
       </c>
@@ -16839,13 +17018,13 @@
         </is>
       </c>
       <c r="D210" s="4" t="n">
-        <v>5.53939307843699</v>
+        <v>5.53959826360174</v>
       </c>
       <c r="E210" s="4" t="n">
-        <v>1.85467070710895e-06</v>
+        <v>1.85170297004909e-06</v>
       </c>
       <c r="F210" s="4" t="n">
-        <v>1.7545460823256e-05</v>
+        <v>1.75320615762131e-05</v>
       </c>
       <c r="G210" s="4" t="b">
         <v>1</v>
@@ -16871,13 +17050,13 @@
         </is>
       </c>
       <c r="D211" s="4" t="n">
-        <v>1.43478024952675</v>
+        <v>1.43477431913659</v>
       </c>
       <c r="E211" s="4" t="n">
-        <v>0.0881202978323723</v>
+        <v>0.0881281064980647</v>
       </c>
       <c r="F211" s="4" t="n">
-        <v>0.128530672065721</v>
+        <v>0.128530923651136</v>
       </c>
       <c r="G211" s="4" t="b">
         <v>1</v>
@@ -16935,13 +17114,13 @@
         </is>
       </c>
       <c r="D213" s="4" t="n">
-        <v>2.88190523363686</v>
+        <v>2.88205898836242</v>
       </c>
       <c r="E213" s="4" t="n">
-        <v>1.04939957631298e-06</v>
+        <v>1.04801792668243e-06</v>
       </c>
       <c r="F213" s="4" t="n">
-        <v>8.5089561260847e-06</v>
+        <v>8.500306179997969e-06</v>
       </c>
       <c r="G213" s="4" t="b">
         <v>1</v>
@@ -16999,13 +17178,13 @@
         </is>
       </c>
       <c r="D215" s="4" t="n">
-        <v>6.30648245228024</v>
+        <v>6.30656875930276</v>
       </c>
       <c r="E215" s="4" t="n">
-        <v>5.560599802299899e-12</v>
+        <v>5.534097654566679e-12</v>
       </c>
       <c r="F215" s="4" t="n">
-        <v>2.97050435094872e-11</v>
+        <v>2.95950416950836e-11</v>
       </c>
       <c r="G215" s="4" t="b">
         <v>1</v>
@@ -17247,13 +17426,13 @@
         </is>
       </c>
       <c r="D223" s="4" t="n">
-        <v>-3.60257957999715</v>
+        <v>-3.60254904086979</v>
       </c>
       <c r="E223" s="4" t="n">
-        <v>3.12138839441096e-06</v>
+        <v>3.1244607313258e-06</v>
       </c>
       <c r="F223" s="4" t="n">
-        <v>2.63504973798448e-05</v>
+        <v>2.63698562575592e-05</v>
       </c>
       <c r="G223" s="4" t="b">
         <v>1</v>
@@ -17279,13 +17458,13 @@
         </is>
       </c>
       <c r="D224" s="4" t="n">
-        <v>3.87027366453888</v>
+        <v>3.87027031505358</v>
       </c>
       <c r="E224" s="4" t="n">
-        <v>1.03913191173216e-10</v>
+        <v>1.0395484735356e-10</v>
       </c>
       <c r="F224" s="4" t="n">
-        <v>2.01791840254862e-09</v>
+        <v>2.02217251957642e-09</v>
       </c>
       <c r="G224" s="4" t="b">
         <v>1</v>
@@ -17343,13 +17522,13 @@
         </is>
       </c>
       <c r="D226" s="4" t="n">
-        <v>1.51853269744947</v>
+        <v>1.51867264246545</v>
       </c>
       <c r="E226" s="4" t="n">
-        <v>0.0031072258414224</v>
+        <v>0.0030957290038751</v>
       </c>
       <c r="F226" s="4" t="n">
-        <v>0.0075203789952188</v>
+        <v>0.0074961670679288</v>
       </c>
       <c r="G226" s="4" t="b">
         <v>1</v>
@@ -17407,13 +17586,13 @@
         </is>
       </c>
       <c r="D228" s="4" t="n">
-        <v>0.89453255383055</v>
+        <v>0.894486382136331</v>
       </c>
       <c r="E228" s="4" t="n">
-        <v>0.0194193753110822</v>
+        <v>0.0194230903956726</v>
       </c>
       <c r="F228" s="4" t="n">
-        <v>0.0282086724890446</v>
+        <v>0.0282069398307599</v>
       </c>
       <c r="G228" s="4" t="b">
         <v>1</v>
@@ -17655,13 +17834,13 @@
         </is>
       </c>
       <c r="D236" s="4" t="n">
-        <v>1.02480786364073</v>
+        <v>1.02489692053288</v>
       </c>
       <c r="E236" s="4" t="n">
-        <v>0.0473560640186704</v>
+        <v>0.0473533837957725</v>
       </c>
       <c r="F236" s="4" t="n">
-        <v>0.0799855197598337</v>
+        <v>0.0799837862690996</v>
       </c>
       <c r="G236" s="4" t="b">
         <v>1</v>
@@ -17687,13 +17866,13 @@
         </is>
       </c>
       <c r="D237" s="4" t="n">
-        <v>7.34274811127424</v>
+        <v>7.34269626558757</v>
       </c>
       <c r="E237" s="4" t="n">
-        <v>1.57217800387344e-06</v>
+        <v>1.57073442221733e-06</v>
       </c>
       <c r="F237" s="4" t="n">
-        <v>8.09649956829022e-06</v>
+        <v>8.095114880650301e-06</v>
       </c>
       <c r="G237" s="4" t="b">
         <v>1</v>
@@ -17751,13 +17930,13 @@
         </is>
       </c>
       <c r="D239" s="4" t="n">
-        <v>3.70101476074938</v>
+        <v>3.70116329657432</v>
       </c>
       <c r="E239" s="4" t="n">
-        <v>2.43360364776657e-07</v>
+        <v>2.42768961665977e-07</v>
       </c>
       <c r="F239" s="4" t="n">
-        <v>2.57969736993345e-06</v>
+        <v>2.57420145817475e-06</v>
       </c>
       <c r="G239" s="4" t="b">
         <v>1</v>
@@ -17815,13 +17994,13 @@
         </is>
       </c>
       <c r="D241" s="4" t="n">
-        <v>1.51085977279679</v>
+        <v>1.51087157558476</v>
       </c>
       <c r="E241" s="4" t="n">
-        <v>0.001401194065142</v>
+        <v>0.0014011260436363</v>
       </c>
       <c r="F241" s="4" t="n">
-        <v>0.0024078517284058</v>
+        <v>0.0024077094059026</v>
       </c>
       <c r="G241" s="4" t="b">
         <v>1</v>
@@ -18063,13 +18242,13 @@
         </is>
       </c>
       <c r="D249" s="4" t="n">
-        <v>-3.86940889072015</v>
+        <v>-3.86922167095915</v>
       </c>
       <c r="E249" s="4" t="n">
-        <v>7.750892548430649e-08</v>
+        <v>7.74612610974429e-08</v>
       </c>
       <c r="F249" s="4" t="n">
-        <v>1.46183147174004e-06</v>
+        <v>1.46126073900769e-06</v>
       </c>
       <c r="G249" s="4" t="b">
         <v>1</v>
@@ -18095,13 +18274,13 @@
         </is>
       </c>
       <c r="D250" s="4" t="n">
-        <v>-3.92423482458367</v>
+        <v>-3.92420100581603</v>
       </c>
       <c r="E250" s="4" t="n">
-        <v>6.954897163013059e-11</v>
+        <v>7.005795652605709e-11</v>
       </c>
       <c r="F250" s="4" t="n">
-        <v>1.42675840837932e-09</v>
+        <v>1.43777814493641e-09</v>
       </c>
       <c r="G250" s="4" t="b">
         <v>1</v>
@@ -18159,13 +18338,13 @@
         </is>
       </c>
       <c r="D252" s="4" t="n">
-        <v>-3.26028228192782</v>
+        <v>-3.26012809409324</v>
       </c>
       <c r="E252" s="4" t="n">
-        <v>3.500304750648619e-11</v>
+        <v>3.48794169937469e-11</v>
       </c>
       <c r="F252" s="4" t="n">
-        <v>2.59581505130507e-09</v>
+        <v>2.59184850955319e-09</v>
       </c>
       <c r="G252" s="4" t="b">
         <v>1</v>
@@ -18223,13 +18402,13 @@
         </is>
       </c>
       <c r="D254" s="4" t="n">
-        <v>2.10989447178502</v>
+        <v>2.10989328284868</v>
       </c>
       <c r="E254" s="4" t="n">
-        <v>2.88137668850818e-25</v>
+        <v>2.87661798981466e-25</v>
       </c>
       <c r="F254" s="4" t="n">
-        <v>1.66711463835891e-23</v>
+        <v>1.66492760111281e-23</v>
       </c>
       <c r="G254" s="4" t="b">
         <v>1</v>
@@ -18471,13 +18650,13 @@
         </is>
       </c>
       <c r="D262" s="4" t="n">
-        <v>0.149840629269991</v>
+        <v>0.149968109032455</v>
       </c>
       <c r="E262" s="4" t="n">
-        <v>0.346385748630503</v>
+        <v>0.346030520762706</v>
       </c>
       <c r="F262" s="4" t="n">
-        <v>0.429969453295509</v>
+        <v>0.429505228531558</v>
       </c>
       <c r="G262" s="4" t="b">
         <v>1</v>
@@ -18503,13 +18682,13 @@
         </is>
       </c>
       <c r="D263" s="4" t="n">
-        <v>-0.243976421699182</v>
+        <v>-0.243992816272735</v>
       </c>
       <c r="E263" s="4" t="n">
-        <v>0.162443531840294</v>
+        <v>0.162408093315816</v>
       </c>
       <c r="F263" s="4" t="n">
-        <v>0.219644862544528</v>
+        <v>0.219605650921876</v>
       </c>
       <c r="G263" s="4" t="b">
         <v>1</v>
@@ -18567,13 +18746,13 @@
         </is>
       </c>
       <c r="D265" s="4" t="n">
-        <v>0.828289025824796</v>
+        <v>0.828447059810231</v>
       </c>
       <c r="E265" s="4" t="n">
-        <v>4.52223073378344e-07</v>
+        <v>4.50053611797464e-07</v>
       </c>
       <c r="F265" s="4" t="n">
-        <v>4.27924520181896e-06</v>
+        <v>4.25999573697131e-06</v>
       </c>
       <c r="G265" s="4" t="b">
         <v>1</v>
@@ -18625,13 +18804,13 @@
         </is>
       </c>
       <c r="D267" s="4" t="n">
-        <v>-0.200608496306742</v>
+        <v>-0.200613623140581</v>
       </c>
       <c r="E267" s="4" t="n">
-        <v>0.0597691631926591</v>
+        <v>0.0597615662784979</v>
       </c>
       <c r="F267" s="4" t="n">
-        <v>0.079764586113269</v>
+        <v>0.07974537404558379</v>
       </c>
       <c r="G267" s="4" t="b">
         <v>1</v>
@@ -18865,13 +19044,13 @@
         </is>
       </c>
       <c r="D275" s="4" t="n">
-        <v>1.11085002609987</v>
+        <v>1.11104750954133</v>
       </c>
       <c r="E275" s="4" t="n">
-        <v>0.0687794893992071</v>
+        <v>0.0687224435663904</v>
       </c>
       <c r="F275" s="4" t="n">
-        <v>0.109923701011085</v>
+        <v>0.109847345393616</v>
       </c>
       <c r="G275" s="4" t="b">
         <v>1</v>
@@ -18897,13 +19076,13 @@
         </is>
       </c>
       <c r="D276" s="4" t="n">
-        <v>3.31231450153575</v>
+        <v>3.31232048653738</v>
       </c>
       <c r="E276" s="4" t="n">
-        <v>0.0003725471598336</v>
+        <v>0.0003733577075165</v>
       </c>
       <c r="F276" s="4" t="n">
-        <v>0.0009932371007792</v>
+        <v>0.0009952647840177</v>
       </c>
       <c r="G276" s="4" t="b">
         <v>1</v>
@@ -18961,13 +19140,13 @@
         </is>
       </c>
       <c r="D278" s="4" t="n">
-        <v>6.29061139755916</v>
+        <v>6.29074669509587</v>
       </c>
       <c r="E278" s="4" t="n">
-        <v>1.31881928574065e-07</v>
+        <v>1.32165655998517e-07</v>
       </c>
       <c r="F278" s="4" t="n">
-        <v>1.5511272058614e-06</v>
+        <v>1.55218889469864e-06</v>
       </c>
       <c r="G278" s="4" t="b">
         <v>1</v>
@@ -19019,13 +19198,13 @@
         </is>
       </c>
       <c r="D280" s="4" t="n">
-        <v>-1.80161423745876</v>
+        <v>-1.8017842856446</v>
       </c>
       <c r="E280" s="4" t="n">
-        <v>1.87116695254079e-07</v>
+        <v>1.86517606975595e-07</v>
       </c>
       <c r="F280" s="4" t="n">
-        <v>5.3261029507146e-07</v>
+        <v>5.31188558726892e-07</v>
       </c>
       <c r="G280" s="4" t="b">
         <v>1</v>
@@ -19267,13 +19446,13 @@
         </is>
       </c>
       <c r="D288" s="4" t="n">
-        <v>0.202491617283925</v>
+        <v>0.202515038912181</v>
       </c>
       <c r="E288" s="4" t="n">
-        <v>0.609769014923418</v>
+        <v>0.6097671484557859</v>
       </c>
       <c r="F288" s="4" t="n">
-        <v>0.680458688502382</v>
+        <v>0.68045703595066</v>
       </c>
       <c r="G288" s="4" t="b">
         <v>1</v>
@@ -19299,13 +19478,13 @@
         </is>
       </c>
       <c r="D289" s="4" t="n">
-        <v>5.80090056105349</v>
+        <v>5.80088197787464</v>
       </c>
       <c r="E289" s="4" t="n">
-        <v>4.3080920664562e-12</v>
+        <v>4.31096352361283e-12</v>
       </c>
       <c r="F289" s="4" t="n">
-        <v>1.29277434766857e-10</v>
+        <v>1.2941564541711e-10</v>
       </c>
       <c r="G289" s="4" t="b">
         <v>1</v>
@@ -19363,13 +19542,13 @@
         </is>
       </c>
       <c r="D291" s="4" t="n">
-        <v>0.0111910412200248</v>
+        <v>0.0113351436376436</v>
       </c>
       <c r="E291" s="4" t="n">
-        <v>0.96726624656583</v>
+        <v>0.966846979887741</v>
       </c>
       <c r="F291" s="4" t="n">
-        <v>0.975693825803277</v>
+        <v>0.975342226794799</v>
       </c>
       <c r="G291" s="4" t="b">
         <v>1</v>
@@ -19427,13 +19606,13 @@
         </is>
       </c>
       <c r="D293" s="4" t="n">
-        <v>0.306216610417165</v>
+        <v>0.306195593824713</v>
       </c>
       <c r="E293" s="4" t="n">
-        <v>0.245848928862128</v>
+        <v>0.245871407563345</v>
       </c>
       <c r="F293" s="4" t="n">
-        <v>0.291959261297603</v>
+        <v>0.291967331388427</v>
       </c>
       <c r="G293" s="4" t="b">
         <v>1</v>
@@ -19675,13 +19854,13 @@
         </is>
       </c>
       <c r="D301" s="4" t="n">
-        <v>-5.8201708107557</v>
+        <v>-5.81972084226626</v>
       </c>
       <c r="E301" s="4" t="n">
-        <v>1.17555758270226e-08</v>
+        <v>1.16918439346725e-08</v>
       </c>
       <c r="F301" s="4" t="n">
-        <v>3.45944251279853e-07</v>
+        <v>3.45287490528439e-07</v>
       </c>
       <c r="G301" s="4" t="b">
         <v>1</v>
@@ -19707,13 +19886,13 @@
         </is>
       </c>
       <c r="D302" s="4" t="n">
-        <v>-4.25910213294597</v>
+        <v>-4.25893483917888</v>
       </c>
       <c r="E302" s="4" t="n">
-        <v>3.0169284166701e-15</v>
+        <v>3.064475452387271e-15</v>
       </c>
       <c r="F302" s="4" t="n">
-        <v>2.13243935574492e-13</v>
+        <v>2.16691818718569e-13</v>
       </c>
       <c r="G302" s="4" t="b">
         <v>1</v>
@@ -19770,9 +19949,15 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D304" s="4" t="n"/>
-      <c r="E304" s="4" t="n"/>
-      <c r="F304" s="4" t="n"/>
+      <c r="D304" s="4" t="n">
+        <v>-1.23905030270118</v>
+      </c>
+      <c r="E304" s="4" t="n">
+        <v>0.368216216655128</v>
+      </c>
+      <c r="F304" s="4" t="n">
+        <v>0.453603142485708</v>
+      </c>
       <c r="G304" s="4" t="b">
         <v>1</v>
       </c>
@@ -19829,13 +20014,13 @@
         </is>
       </c>
       <c r="D306" s="4" t="n">
-        <v>2.79300302421463</v>
+        <v>2.7931180108718</v>
       </c>
       <c r="E306" s="4" t="n">
-        <v>3.00157626785448e-10</v>
+        <v>2.99374525467797e-10</v>
       </c>
       <c r="F306" s="4" t="n">
-        <v>1.23803437643529e-09</v>
+        <v>1.23522450151616e-09</v>
       </c>
       <c r="G306" s="4" t="b">
         <v>1</v>
@@ -20077,13 +20262,13 @@
         </is>
       </c>
       <c r="D314" s="4" t="n">
-        <v>0.456223111436911</v>
+        <v>0.456259459672538</v>
       </c>
       <c r="E314" s="4" t="n">
-        <v>0.589326718247022</v>
+        <v>0.589300566542077</v>
       </c>
       <c r="F314" s="4" t="n">
-        <v>0.662104681748594</v>
+        <v>0.6620151708920839</v>
       </c>
       <c r="G314" s="4" t="b">
         <v>1</v>
@@ -20109,13 +20294,13 @@
         </is>
       </c>
       <c r="D315" s="4" t="n">
-        <v>3.83214790364178</v>
+        <v>3.83213720735594</v>
       </c>
       <c r="E315" s="4" t="n">
-        <v>1.42362661299867e-05</v>
+        <v>1.42589837918451e-05</v>
       </c>
       <c r="F315" s="4" t="n">
-        <v>5.53059841267574e-05</v>
+        <v>5.54165246611952e-05</v>
       </c>
       <c r="G315" s="4" t="b">
         <v>1</v>
@@ -20172,14 +20357,20 @@
           <t>M</t>
         </is>
       </c>
-      <c r="D317" s="4" t="n"/>
-      <c r="E317" s="4" t="n"/>
-      <c r="F317" s="4" t="n"/>
+      <c r="D317" s="4" t="n">
+        <v>7.1818652574327</v>
+      </c>
+      <c r="E317" s="4" t="n">
+        <v>0.0002188949595165</v>
+      </c>
+      <c r="F317" s="4" t="n">
+        <v>0.0007585852383143</v>
+      </c>
       <c r="G317" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H317" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="318">
@@ -20231,13 +20422,13 @@
         </is>
       </c>
       <c r="D319" s="4" t="n">
-        <v>1.07357998097036</v>
+        <v>1.07358920166374</v>
       </c>
       <c r="E319" s="4" t="n">
-        <v>0.0078012924588847</v>
+        <v>0.0078001637012007</v>
       </c>
       <c r="F319" s="4" t="n">
-        <v>0.0120441006382782</v>
+        <v>0.0120401308873742</v>
       </c>
       <c r="G319" s="4" t="b">
         <v>1</v>
@@ -20557,13 +20748,13 @@
         </is>
       </c>
       <c r="D330" s="4" t="n">
-        <v>-6.51078191974072</v>
+        <v>-6.51065647039742</v>
       </c>
       <c r="E330" s="4" t="n">
-        <v>6.29183113993787e-07</v>
+        <v>6.31602454780881e-07</v>
       </c>
       <c r="F330" s="4" t="n">
-        <v>5.5745161670559e-06</v>
+        <v>5.59659447290205e-06</v>
       </c>
       <c r="G330" s="4" t="b">
         <v>1</v>
@@ -20823,13 +21014,13 @@
         </is>
       </c>
       <c r="D340" s="4" t="n">
-        <v>-5.05271659215968</v>
+        <v>-5.05268553050679</v>
       </c>
       <c r="E340" s="4" t="n">
-        <v>2.68730010763004e-06</v>
+        <v>2.68660934474157e-06</v>
       </c>
       <c r="F340" s="4" t="n">
-        <v>2.35224636756368e-05</v>
+        <v>2.35101421185051e-05</v>
       </c>
       <c r="G340" s="4" t="b">
         <v>1</v>
@@ -20855,13 +21046,13 @@
         </is>
       </c>
       <c r="D341" s="4" t="n">
-        <v>0.168028315316068</v>
+        <v>0.16796539593541</v>
       </c>
       <c r="E341" s="4" t="n">
-        <v>0.805738855562671</v>
+        <v>0.8058374365555711</v>
       </c>
       <c r="F341" s="4" t="n">
-        <v>0.845776273357381</v>
+        <v>0.845862850246878</v>
       </c>
       <c r="G341" s="4" t="b">
         <v>1</v>
@@ -20919,13 +21110,13 @@
         </is>
       </c>
       <c r="D343" s="4" t="n">
-        <v>2.7924588510941</v>
+        <v>2.79261338602242</v>
       </c>
       <c r="E343" s="4" t="n">
-        <v>4.10768807379545e-12</v>
+        <v>4.09917074768716e-12</v>
       </c>
       <c r="F343" s="4" t="n">
-        <v>5.15941122778421e-10</v>
+        <v>5.15026000166958e-10</v>
       </c>
       <c r="G343" s="4" t="b">
         <v>1</v>
@@ -20983,13 +21174,13 @@
         </is>
       </c>
       <c r="D345" s="4" t="n">
-        <v>-2.35874899425477</v>
+        <v>-2.35876804118651</v>
       </c>
       <c r="E345" s="4" t="n">
-        <v>2.728338509576629e-16</v>
+        <v>2.72651423467015e-16</v>
       </c>
       <c r="F345" s="4" t="n">
-        <v>2.80978715744486e-15</v>
+        <v>2.80784338617144e-15</v>
       </c>
       <c r="G345" s="4" t="b">
         <v>1</v>
@@ -21231,13 +21422,13 @@
         </is>
       </c>
       <c r="D353" s="4" t="n">
-        <v>-1.07314818313707</v>
+        <v>-1.07312819734049</v>
       </c>
       <c r="E353" s="4" t="n">
-        <v>0.0371518334988072</v>
+        <v>0.0371727495001763</v>
       </c>
       <c r="F353" s="4" t="n">
-        <v>0.0648926953411913</v>
+        <v>0.0649310763216419</v>
       </c>
       <c r="G353" s="4" t="b">
         <v>1</v>
@@ -21263,13 +21454,13 @@
         </is>
       </c>
       <c r="D354" s="4" t="n">
-        <v>0.879660525837475</v>
+        <v>0.87963365861819</v>
       </c>
       <c r="E354" s="4" t="n">
-        <v>0.0189602578139942</v>
+        <v>0.0189723938480236</v>
       </c>
       <c r="F354" s="4" t="n">
-        <v>0.0330961241851486</v>
+        <v>0.0331151282419879</v>
       </c>
       <c r="G354" s="4" t="b">
         <v>1</v>
@@ -21327,13 +21518,13 @@
         </is>
       </c>
       <c r="D356" s="4" t="n">
-        <v>-0.0735939334740687</v>
+        <v>-0.0734359228748238</v>
       </c>
       <c r="E356" s="4" t="n">
-        <v>0.550975383742533</v>
+        <v>0.551835951348236</v>
       </c>
       <c r="F356" s="4" t="n">
-        <v>0.631135357407562</v>
+        <v>0.631999240664361</v>
       </c>
       <c r="G356" s="4" t="b">
         <v>1</v>
@@ -21391,13 +21582,13 @@
         </is>
       </c>
       <c r="D358" s="4" t="n">
-        <v>0.489424717717857</v>
+        <v>0.489423281916906</v>
       </c>
       <c r="E358" s="4" t="n">
-        <v>0.0045040967367715</v>
+        <v>0.0045036615454324</v>
       </c>
       <c r="F358" s="4" t="n">
-        <v>0.0071971518586055</v>
+        <v>0.0071949933035646</v>
       </c>
       <c r="G358" s="4" t="b">
         <v>1</v>
@@ -21638,9 +21829,15 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D366" s="4" t="n"/>
-      <c r="E366" s="4" t="n"/>
-      <c r="F366" s="4" t="n"/>
+      <c r="D366" s="4" t="n">
+        <v>-4.56972967374015</v>
+      </c>
+      <c r="E366" s="4" t="n">
+        <v>2.67132986713465e-06</v>
+      </c>
+      <c r="F366" s="4" t="n">
+        <v>2.33994305331696e-05</v>
+      </c>
       <c r="G366" s="4" t="b">
         <v>1</v>
       </c>
@@ -21664,9 +21861,15 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D367" s="4" t="n"/>
-      <c r="E367" s="4" t="n"/>
-      <c r="F367" s="4" t="n"/>
+      <c r="D367" s="4" t="n">
+        <v>0.396082184030924</v>
+      </c>
+      <c r="E367" s="4" t="n">
+        <v>0.706856956233779</v>
+      </c>
+      <c r="F367" s="4" t="n">
+        <v>0.76311908733777</v>
+      </c>
       <c r="G367" s="4" t="b">
         <v>1</v>
       </c>
@@ -21723,13 +21926,13 @@
         </is>
       </c>
       <c r="D369" s="4" t="n">
-        <v>-2.82879105446469</v>
+        <v>-2.8286472909554</v>
       </c>
       <c r="E369" s="4" t="n">
-        <v>2.28150944916731e-06</v>
+        <v>2.2820310869899e-06</v>
       </c>
       <c r="F369" s="4" t="n">
-        <v>1.60889919524436e-05</v>
+        <v>1.60975053053663e-05</v>
       </c>
       <c r="G369" s="4" t="b">
         <v>1</v>
@@ -21787,13 +21990,13 @@
         </is>
       </c>
       <c r="D371" s="4" t="n">
-        <v>12.3327491631417</v>
+        <v>12.332736329799</v>
       </c>
       <c r="E371" s="4" t="n">
-        <v>3.986399857367541e-15</v>
+        <v>3.958356067867411e-15</v>
       </c>
       <c r="F371" s="4" t="n">
-        <v>3.34003034799734e-14</v>
+        <v>3.31766206121544e-14</v>
       </c>
       <c r="G371" s="4" t="b">
         <v>1</v>
@@ -22029,13 +22232,13 @@
         </is>
       </c>
       <c r="D379" s="4" t="n">
-        <v>1.97755952698707</v>
+        <v>1.97779580453918</v>
       </c>
       <c r="E379" s="4" t="n">
-        <v>0.0012240822891056</v>
+        <v>0.0012231155249824</v>
       </c>
       <c r="F379" s="4" t="n">
-        <v>0.0035645340325869</v>
+        <v>0.0035608967756441</v>
       </c>
       <c r="G379" s="4" t="b">
         <v>1</v>
@@ -22060,14 +22263,20 @@
           <t>H</t>
         </is>
       </c>
-      <c r="D380" s="4" t="n"/>
-      <c r="E380" s="4" t="n"/>
-      <c r="F380" s="4" t="n"/>
+      <c r="D380" s="4" t="n">
+        <v>5.76204493814367</v>
+      </c>
+      <c r="E380" s="4" t="n">
+        <v>2.53746331990421e-05</v>
+      </c>
+      <c r="F380" s="4" t="n">
+        <v>9.24539051413598e-05</v>
+      </c>
       <c r="G380" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H380" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="381">
@@ -22119,13 +22328,13 @@
         </is>
       </c>
       <c r="D382" s="4" t="n">
-        <v>-4.96572267222828</v>
+        <v>-4.96557617433502</v>
       </c>
       <c r="E382" s="4" t="n">
-        <v>7.746094418642749e-12</v>
+        <v>7.725598798043599e-12</v>
       </c>
       <c r="F382" s="4" t="n">
-        <v>8.12059063699288e-10</v>
+        <v>8.101537385223991e-10</v>
       </c>
       <c r="G382" s="4" t="b">
         <v>1</v>
@@ -22182,14 +22391,20 @@
           <t>C</t>
         </is>
       </c>
-      <c r="D384" s="4" t="n"/>
-      <c r="E384" s="4" t="n"/>
-      <c r="F384" s="4" t="n"/>
+      <c r="D384" s="4" t="n">
+        <v>7.8864207705603</v>
+      </c>
+      <c r="E384" s="4" t="n">
+        <v>1.19426735561224e-05</v>
+      </c>
+      <c r="F384" s="4" t="n">
+        <v>2.72031676399992e-05</v>
+      </c>
       <c r="G384" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H384" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="385">
@@ -22413,13 +22628,13 @@
         </is>
       </c>
       <c r="D392" s="4" t="n">
-        <v>-2.681023923876</v>
+        <v>-2.68086692647017</v>
       </c>
       <c r="E392" s="4" t="n">
-        <v>1.10334426330144e-07</v>
+        <v>1.10442428171174e-07</v>
       </c>
       <c r="F392" s="4" t="n">
-        <v>1.93270523715853e-06</v>
+        <v>1.93388275405336e-06</v>
       </c>
       <c r="G392" s="4" t="b">
         <v>1</v>
@@ -22445,13 +22660,13 @@
         </is>
       </c>
       <c r="D393" s="4" t="n">
-        <v>-0.297043596933865</v>
+        <v>-0.296944271073459</v>
       </c>
       <c r="E393" s="4" t="n">
-        <v>0.290266895723539</v>
+        <v>0.290540587696088</v>
       </c>
       <c r="F393" s="4" t="n">
-        <v>0.360693258025401</v>
+        <v>0.360987092792626</v>
       </c>
       <c r="G393" s="4" t="b">
         <v>1</v>
@@ -22509,13 +22724,13 @@
         </is>
       </c>
       <c r="D395" s="4" t="n">
-        <v>0.0482998881432219</v>
+        <v>0.0484550455320749</v>
       </c>
       <c r="E395" s="4" t="n">
-        <v>0.850818314935522</v>
+        <v>0.850352940135113</v>
       </c>
       <c r="F395" s="4" t="n">
-        <v>0.888802852839732</v>
+        <v>0.888444375674232</v>
       </c>
       <c r="G395" s="4" t="b">
         <v>1</v>
@@ -22567,13 +22782,13 @@
         </is>
       </c>
       <c r="D397" s="4" t="n">
-        <v>-0.236428784750778</v>
+        <v>-0.236448647804827</v>
       </c>
       <c r="E397" s="4" t="n">
-        <v>0.184853802115731</v>
+        <v>0.184809717409809</v>
       </c>
       <c r="F397" s="4" t="n">
-        <v>0.225201979266582</v>
+        <v>0.225131559135034</v>
       </c>
       <c r="G397" s="4" t="b">
         <v>1</v>
@@ -22809,7 +23024,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22881,7 +23096,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>GSE230581 log2FC &gt;= 0.5 &amp; FDR &lt; 0.05; NE if no orthologue / not measured</t>
+          <t>GSE230581 log2FC &gt;= 0.5 &amp; FDR &lt; 0.05; zero_expression = fail; NE only for no_1to1_orthologue / not_available_in_source</t>
         </is>
       </c>
     </row>
@@ -22958,7 +23173,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>HGCA &gt;=9 PCW &amp; GSE230581 &amp; Joanito &amp; Pelka each log2FC &gt;= 0.5 &amp; FDR &lt; 0.05 (not measured = NE)</t>
+          <t>HGCA &gt;=9 PCW &amp; GSE230581 &amp; Joanito &amp; Pelka each log2FC &gt;= 0.5 &amp; FDR &lt; 0.05 (panel-aware values; NA only with an explicit NA_reason)</t>
         </is>
       </c>
     </row>
@@ -22971,22 +23186,39 @@
       <c r="B10" s="4" t="inlineStr"/>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>log2FC (FDR); ** log2FC &gt;= 0.5 &amp; FDR &lt; 0.05; * FDR &lt; 0.05 below effect threshold; NA = not measured / no orthologue</t>
+          <t>log2FC (FDR); ** log2FC &gt;= 0.5 &amp; FDR &lt; 0.05; * FDR &lt; 0.05 below effect threshold; [low count] = mean CPM &lt; 1 in both arms; NA (reason) uses the fixed NA vocabulary</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>Panel-gene evaluation</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>data-QC amendment</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>gate contrasts re-run with the 31 panel genes exempt from filterByExpr (any counts kept); zero counts in all samples = zero_expression (evaluable, no enrichment)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Supportive evidence</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>never selecting</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>GSE44433, TCGA, Pikkupeura cultures, HGCA all fetal, Joanito sensitivity, Pelka P</t>
         </is>

</xml_diff>